<commit_message>
docs: v0.2.0 release notes, README and refreshed media
Resolves the open question on the federal 50% agentic-AI target with
the Cabinet announcement.
</commit_message>
<xml_diff>
--- a/public/templates/ar/control-checklist.xlsx
+++ b/public/templates/ar/control-checklist.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J58"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -521,7 +521,7 @@
         <v>تعيين مالك أعمال محدد بالاسم لكل حالة استخدام يتحمّل المسؤولية عن نتائجها، وتوثيق جهات الاتصال التقنية ومسؤولي البيانات والمخاطر المرتبطين بها.</v>
       </c>
       <c r="E4" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Governance and accountability; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.3.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.1</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Governance and accountability; كود الإمارات للخدمات الحكومية: Agentic Reference p.9; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.3.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.1</v>
       </c>
       <c r="F4" t="str">
         <v>بحاجة إلى تحقق</v>
@@ -617,7 +617,7 @@
         <v>اشتراط قرار موثّق بالإطلاق أو عدمه من لجنة أو مسؤول مخوّل قبل تشغيل أي نظام عالي المخاطر، بناءً على نتائج الاختبار والمخاطر المتبقية.</v>
       </c>
       <c r="E7" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 1.1, GOVERN 2.3</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1, Code 8.8, Agentic Guide §06; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 1.1, GOVERN 2.3</v>
       </c>
       <c r="F7" t="str">
         <v>تم التحقق</v>
@@ -681,7 +681,7 @@
         <v>تدريب الموظفين الذين يطوّرون أنظمة الذكاء الاصطناعي أو يشغّلونها أو يعتمدون عليها على قدراتها وحدودها وعلى مسؤولياتهم، بما يتناسب مع أدوارهم.</v>
       </c>
       <c r="E9" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Promoting AI awareness for an inclusive society; آيزو/آي إي سي 42001: A.4.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.2, MAP 3.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 4</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Promoting AI awareness for an inclusive society; كود الإمارات للخدمات الحكومية: Code 6.2; آيزو/آي إي سي 42001: A.4.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.2, MAP 3.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 4</v>
       </c>
       <c r="F9" t="str">
         <v>بحاجة إلى تحقق</v>
@@ -733,25 +733,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>CTL-TRA-01</v>
+        <v>CTL-ACC-09</v>
       </c>
       <c r="B11" t="str">
-        <v>الشفافية</v>
+        <v>المساءلة</v>
       </c>
       <c r="C11" t="str">
-        <v>الإفصاح عن التعامل مع الذكاء الاصطناعي</v>
+        <v>مراجعة حوكمة لكل وكيل</v>
       </c>
       <c r="D11" t="str">
-        <v>إبلاغ الأشخاص بوضوح، منذ بداية التفاعل، بأنهم يتعاملون مع نظام ذكاء اصطناعي وليس مع موظف بشري.</v>
+        <v>إجراء مراجعة حوكمة موثقة لكل وكيل ذكاء اصطناعي قبل إطلاقه، وإعادتها عند أي تغيير في نطاقه أو صلاحياته أو بياناته أو مخرجاته، مع تسجيل كل قرار بالاستمرار أو التعديل أو الإيقاف في سجل مراجعة خاص بالوكيل.</v>
       </c>
       <c r="E11" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Transparency; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 50</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1, Agentic Guide §06; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 1.1</v>
       </c>
       <c r="F11" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G11" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -765,25 +765,25 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CTL-TRA-02</v>
+        <v>CTL-ACC-10</v>
       </c>
       <c r="B12" t="str">
-        <v>الشفافية</v>
+        <v>المساءلة</v>
       </c>
       <c r="C12" t="str">
-        <v>وسم المحتوى المُنشأ بالذكاء الاصطناعي</v>
+        <v>وثيقة نطاق معتمدة لكل وكيل</v>
       </c>
       <c r="D12" t="str">
-        <v>وسم النصوص والصور والمقاطع الصوتية أو المرئية المُنتجة بالذكاء الاصطناعي التوليدي بأنها مُنشأة آليًا قبل نشرها أو إرسالها للجمهور.</v>
+        <v>الاحتفاظ لكل وكيل بوثيقة نطاق معتمدة ومحدّثة تحدد الخدمات والحالات التي يجوز له التعامل معها، وصلاحياته وحدود وصوله، والقرارات التي يتخذها بمفرده وتلك التي يجب أن يحيلها إلى موظف، مع إعادة اعتمادها بعد أي تغيير جوهري ومنع تشغيله خارج نطاقها.</v>
       </c>
       <c r="E12" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 50</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.4, Agentic Guide §05; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.3</v>
       </c>
       <c r="F12" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G12" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -797,25 +797,25 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CTL-TRA-03</v>
+        <v>CTL-ACC-11</v>
       </c>
       <c r="B13" t="str">
-        <v>الشفافية</v>
+        <v>المساءلة</v>
       </c>
       <c r="C13" t="str">
-        <v>تقديم التفسير عند الطلب</v>
+        <v>تصنيف الأنظمة وفق التعريف الوطني للذكاء الاصطناعي المساعد</v>
       </c>
       <c r="D13" t="str">
-        <v>توفير وسيلة ميسّرة تتيح للشخص المتأثر بقرار مهم استند إلى الذكاء الاصطناعي طلب تفسير بلغة واضحة للعوامل الرئيسية وراء القرار والحصول عليه.</v>
+        <v>قبل تسجيل أي نظام ذكاء اصطناعي، يُصنَّف توليديًا أو مساعدًا أو متعدد المساعدين وفق التعريف الوطني ومعايير التقييم الذاتي، ولا تُصنَّف روبوتات المحادثة أو الأتمتة المبرمجة مسبقًا أو أدوات صياغة الردود أو الشخصيات الافتراضية أنظمةَ ذكاء اصطناعي مساعد ما لم تستوفِ جميع المعايير.</v>
       </c>
       <c r="E13" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Explainability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.9; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 86</v>
+        <v>كود الإمارات للخدمات الحكومية: Agentic Reference p.6, Agentic Reference p.7, Agentic Reference p.9, Agentic Reference p.13, Agentic Reference p.14; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.1</v>
       </c>
       <c r="F13" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G13" t="str">
-        <v>مخاطر مرتفعة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -829,25 +829,25 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CTL-TRA-04</v>
+        <v>CTL-TRA-01</v>
       </c>
       <c r="B14" t="str">
         <v>الشفافية</v>
       </c>
       <c r="C14" t="str">
-        <v>إخطار الأفراد بالقرارات المدعومة بالذكاء الاصطناعي</v>
+        <v>الإفصاح عن التعامل مع الذكاء الاصطناعي</v>
       </c>
       <c r="D14" t="str">
-        <v>إخطار الأفراد عندما يُتخذ قرار يؤثر فيهم تأثيرًا مهمًا بواسطة نظام ذكاء اصطناعي أو بدعم منه، بمن فيهم الموظفون المتأثرون باستخدامه في بيئة العمل.</v>
+        <v>إبلاغ الأشخاص بوضوح، منذ بداية التفاعل، بأنهم يتعاملون مع نظام ذكاء اصطناعي وليس مع موظف بشري.</v>
       </c>
       <c r="E14" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.5; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Transparency; كود الإمارات للخدمات الحكومية: Code 5.6, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 50</v>
       </c>
       <c r="F14" t="str">
-        <v>تم التحقق</v>
+        <v>بحاجة إلى تحقق</v>
       </c>
       <c r="G14" t="str">
-        <v>مخاطر مرتفعة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H14" t="str">
         <v/>
@@ -861,25 +861,25 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CTL-TRA-05</v>
+        <v>CTL-TRA-02</v>
       </c>
       <c r="B15" t="str">
         <v>الشفافية</v>
       </c>
       <c r="C15" t="str">
-        <v>توثيق النظام</v>
+        <v>وسم المحتوى المُنشأ بالذكاء الاصطناعي</v>
       </c>
       <c r="D15" t="str">
-        <v>الاحتفاظ بتوثيق لكل نظام يشمل الغرض والتصميم والبيانات وإصدار النموذج ونتائج الاختبار والقيود المعروفة، بدرجة تفصيل تمكّن المراجع من فهمه.</v>
+        <v>وسم النصوص والصور والمقاطع الصوتية أو المرئية المُنتجة بالذكاء الاصطناعي التوليدي بأنها مُنشأة آليًا قبل نشرها أو إرسالها للجمهور.</v>
       </c>
       <c r="E15" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety, Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.3, A.6.2.7; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.1, MAP 2.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 11</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 50</v>
       </c>
       <c r="F15" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G15" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H15" t="str">
         <v/>
@@ -893,25 +893,25 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CTL-TRA-06</v>
+        <v>CTL-TRA-03</v>
       </c>
       <c r="B16" t="str">
         <v>الشفافية</v>
       </c>
       <c r="C16" t="str">
-        <v>إفصاح عام عن استخدام الذكاء الاصطناعي</v>
+        <v>تقديم التفسير عند الطلب</v>
       </c>
       <c r="D16" t="str">
-        <v>نشر ملخص بلغة واضحة يبيّن مواضع استخدام الجهة للذكاء الاصطناعي في خدماتها للجمهور، والبيانات التي تعتمد عليها، وطريقة تقديم الملاحظات أو الشكاوى.</v>
+        <v>توفير وسيلة ميسّرة تتيح للشخص المتأثر بقرار مهم استند إلى الذكاء الاصطناعي طلب تفسير بلغة واضحة للعوامل الرئيسية وراء القرار والحصول عليه.</v>
       </c>
       <c r="E16" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 4.2</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Explainability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.9; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 86</v>
       </c>
       <c r="F16" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G16" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر مرتفعة</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -925,25 +925,25 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>CTL-TRA-07</v>
+        <v>CTL-TRA-04</v>
       </c>
       <c r="B17" t="str">
         <v>الشفافية</v>
       </c>
       <c r="C17" t="str">
-        <v>تعليمات الاستخدام للمشغّلين</v>
+        <v>إخطار الأفراد بالقرارات المدعومة بالذكاء الاصطناعي</v>
       </c>
       <c r="D17" t="str">
-        <v>تزويد من يشغّلون النظام أو يعتمدون عليه بتعليمات مكتوبة حول الاستخدام المقصود ومستوى الدقة والقيود والحالات التي لا ينبغي فيها الوثوق بمخرجاته.</v>
+        <v>إخطار الأفراد عندما يُتخذ قرار يؤثر فيهم تأثيرًا مهمًا بواسطة نظام ذكاء اصطناعي أو بدعم منه، بمن فيهم الموظفون المتأثرون باستخدامه في بيئة العمل.</v>
       </c>
       <c r="E17" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 13</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.5; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26</v>
       </c>
       <c r="F17" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G17" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر مرتفعة</v>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -957,25 +957,25 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CTL-DAT-01</v>
+        <v>CTL-TRA-05</v>
       </c>
       <c r="B18" t="str">
-        <v>البيانات</v>
+        <v>الشفافية</v>
       </c>
       <c r="C18" t="str">
-        <v>مصادر البيانات ومنشؤها</v>
+        <v>توثيق النظام</v>
       </c>
       <c r="D18" t="str">
-        <v>توثيق مصدر كل مجموعة بيانات تُستخدم في بناء النظام أو ضبطه أو تشغيله، والحق في استخدامها، وطريقة جمعها وتجهيزها.</v>
+        <v>الاحتفاظ بتوثيق لكل نظام يشمل الغرض والتصميم والبيانات وإصدار النموذج ونتائج الاختبار والقيود المعروفة، بدرجة تفصيل تمكّن المراجع من فهمه.</v>
       </c>
       <c r="E18" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.7.2, A.7.3, A.7.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety, Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.3, A.6.2.7; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.1, MAP 2.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 11</v>
       </c>
       <c r="F18" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G18" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -989,19 +989,19 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CTL-DAT-02</v>
+        <v>CTL-TRA-06</v>
       </c>
       <c r="B19" t="str">
-        <v>البيانات</v>
+        <v>الشفافية</v>
       </c>
       <c r="C19" t="str">
-        <v>جودة البيانات وتمثيلها</v>
+        <v>إفصاح عام عن استخدام الذكاء الاصطناعي</v>
       </c>
       <c r="D19" t="str">
-        <v>التحقق من أن بيانات التدريب والإدخال دقيقة ومكتملة وممثِّلة للفئات التي سيؤثر فيها النظام، وتوثيق عمليات التحقق وأي فجوات.</v>
+        <v>نشر ملخص بلغة واضحة يبيّن مواضع استخدام الجهة للذكاء الاصطناعي في خدماتها للجمهور، والبيانات التي تعتمد عليها، وطريقة تقديم الملاحظات أو الشكاوى.</v>
       </c>
       <c r="E19" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Fairness; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Fairness, Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.7.4, A.7.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 4.2</v>
       </c>
       <c r="F19" t="str">
         <v>تم التحقق</v>
@@ -1021,25 +1021,25 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CTL-DAT-03</v>
+        <v>CTL-TRA-07</v>
       </c>
       <c r="B20" t="str">
-        <v>البيانات</v>
+        <v>الشفافية</v>
       </c>
       <c r="C20" t="str">
-        <v>مراجعة الخصوصية وتقليل البيانات</v>
+        <v>تعليمات الاستخدام للمشغّلين</v>
       </c>
       <c r="D20" t="str">
-        <v>عند استخدام بيانات شخصية، يجب إجراء مراجعة للخصوصية والاقتصار على الحد الأدنى من البيانات الشخصية اللازمة للغرض، بما يتوافق مع سياسة حماية البيانات في الجهة.</v>
+        <v>تزويد من يشغّلون النظام أو يعتمدون عليه بتعليمات مكتوبة حول الاستخدام المقصود ومستوى الدقة والقيود والحالات التي لا ينبغي فيها الوثوق بمخرجاته.</v>
       </c>
       <c r="E20" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Data privacy; أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.2.3, A.7.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.10</v>
+        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 13</v>
       </c>
       <c r="F20" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G20" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -1053,19 +1053,19 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CTL-DAT-04</v>
+        <v>CTL-TRA-08</v>
       </c>
       <c r="B21" t="str">
-        <v>البيانات</v>
+        <v>الشفافية</v>
       </c>
       <c r="C21" t="str">
-        <v>تبرير استخدام السمات الحساسة</v>
+        <v>الإفصاح عن مصادر البيانات التي استخدمها الوكيل</v>
       </c>
       <c r="D21" t="str">
-        <v>عدم استخدام السمات الحساسة أو ما يدل عليها بشكل غير مباشر كمدخلات للنموذج، ما لم يوجد مبرر موثّق ومعتمد مثل اختبار التحيّز.</v>
+        <v>عند تقديم الخدمة عبر وكيل ذكاء اصطناعي، يُوضَّح للمتعامل مصادر البيانات التي اعتمد عليها، ويُبيَّن له قبل التنفيذ أيّ بياناته سيستخدمها الوكيل.</v>
       </c>
       <c r="E21" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Fairness; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Fairness; آيزو/آي إي سي 42001: A.7.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.11; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.2, Agentic Guide §03; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2</v>
       </c>
       <c r="F21" t="str">
         <v>تم التحقق</v>
@@ -1085,22 +1085,22 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CTL-DAT-05</v>
+        <v>CTL-TRA-09</v>
       </c>
       <c r="B22" t="str">
-        <v>البيانات</v>
+        <v>الشفافية</v>
       </c>
       <c r="C22" t="str">
-        <v>اختبار التحيّز والإنصاف</v>
+        <v>إشعار واضح عند تعذّر إكمال الخدمة</v>
       </c>
       <c r="D22" t="str">
-        <v>اختبار النتائج عبر الفئات ذات الصلة قبل الإطلاق وبعد التغييرات الجوهرية، مع تحديد حدّ مقبول مسبقًا، وتوثيق النتائج وأي إجراءات معالجة.</v>
+        <v>إذا تعذّر على الذكاء الاصطناعي إكمال الخدمة، يُبلَّغ المتعامل فورًا وبلغة غير تقنية بسبب التعذّر وبالخطوات التالية، بما في ذلك طريقة التواصل مع موظف.</v>
       </c>
       <c r="E22" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Algorithmic bias; أخلاقيات الذكاء الاصطناعي في دبي: Fairness; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Fairness; آيزو/آي إي سي 42001: A.5.4, A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.11; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 4.5, Agentic Guide §03</v>
       </c>
       <c r="F22" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G22" t="str">
         <v>مخاطر محدودة</v>
@@ -1117,19 +1117,19 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CTL-DAT-06</v>
+        <v>CTL-DAT-01</v>
       </c>
       <c r="B23" t="str">
         <v>البيانات</v>
       </c>
       <c r="C23" t="str">
-        <v>ضوابط إدخال البيانات في أدوات الذكاء الاصطناعي التوليدي</v>
+        <v>مصادر البيانات ومنشؤها</v>
       </c>
       <c r="D23" t="str">
-        <v>وضع قواعد واضحة لنوع المعلومات التي يجوز للموظفين إدخالها في أدوات الذكاء الاصطناعي التوليدي، ومنع إدخال البيانات الشخصية أو الحساسة أو المصنّفة في الخدمات الخارجية إلا بموافقة صريحة.</v>
+        <v>توثيق مصدر كل مجموعة بيانات تُستخدم في بناء النظام أو ضبطه أو تشغيله، والحق في استخدامها، وطريقة جمعها وتجهيزها.</v>
       </c>
       <c r="E23" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.2.3, A.9.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MEASURE 2.10</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.7.2, A.7.3, A.7.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
       </c>
       <c r="F23" t="str">
         <v>تم التحقق</v>
@@ -1149,19 +1149,19 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>CTL-DAT-07</v>
+        <v>CTL-DAT-02</v>
       </c>
       <c r="B24" t="str">
         <v>البيانات</v>
       </c>
       <c r="C24" t="str">
-        <v>حقوق استخدام محتوى التدريب والإسناد</v>
+        <v>جودة البيانات وتمثيلها</v>
       </c>
       <c r="D24" t="str">
-        <v>التأكد من امتلاك الجهة حق استخدام الوثائق والمحتوى المستخدم في تدريب النموذج أو ضبطه أو إسناد إجاباته، والاحتفاظ بسجل لهذا التحقق.</v>
+        <v>التحقق من أن بيانات التدريب والإدخال دقيقة ومكتملة وممثِّلة للفئات التي سيؤثر فيها النظام، وتوثيق عمليات التحقق وأي فجوات.</v>
       </c>
       <c r="E24" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.7.3, A.7.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 4.1, GOVERN 6.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 53</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.3; أخلاقيات الذكاء الاصطناعي في دبي: Fairness; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Fairness, Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.7.4, A.7.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
       </c>
       <c r="F24" t="str">
         <v>تم التحقق</v>
@@ -1181,25 +1181,25 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>CTL-HUM-01</v>
+        <v>CTL-DAT-03</v>
       </c>
       <c r="B25" t="str">
-        <v>الإشراف البشري</v>
+        <v>البيانات</v>
       </c>
       <c r="C25" t="str">
-        <v>نموذج محدد للإشراف البشري</v>
+        <v>مراجعة الخصوصية وتقليل البيانات</v>
       </c>
       <c r="D25" t="str">
-        <v>تحديد وتوثيق مواضع مراجعة البشر لمخرجات النظام أو الموافقة عليها أو مراقبتها لكل حالة استخدام، وإسناد هذا الدور إلى أشخاص يملكون الكفاءة والصلاحية للتدخل.</v>
+        <v>عند استخدام بيانات شخصية، يجب إجراء مراجعة للخصوصية والاقتصار على الحد الأدنى من البيانات الشخصية اللازمة للغرض، بما يتوافق مع سياسة حماية البيانات في الجهة.</v>
       </c>
       <c r="E25" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Human oversight; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.1.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.5, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14, Art. 26</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Data privacy; كود الإمارات للخدمات الحكومية: Code 5.2, Code 5.7, Data Sharing Policy Art. 5; أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.2.3, A.7.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.10</v>
       </c>
       <c r="F25" t="str">
         <v>بحاجة إلى تحقق</v>
       </c>
       <c r="G25" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -1213,19 +1213,19 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>CTL-HUM-02</v>
+        <v>CTL-DAT-04</v>
       </c>
       <c r="B26" t="str">
-        <v>الإشراف البشري</v>
+        <v>البيانات</v>
       </c>
       <c r="C26" t="str">
-        <v>حق الاعتراض على القرار</v>
+        <v>تبرير استخدام السمات الحساسة</v>
       </c>
       <c r="D26" t="str">
-        <v>إتاحة مسار واضح للأفراد للاعتراض على أي قرار مهم استند إلى الذكاء الاصطناعي، ومراجعته من قِبل شخص مخوّل بتعديله.</v>
+        <v>عدم استخدام السمات الحساسة أو ما يدل عليها بشكل غير مباشر كمدخلات للنموذج، ما لم يوجد مبرر موثّق ومعتمد مثل اختبار التحيّز.</v>
       </c>
       <c r="E26" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 3.3</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Fairness; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Fairness; آيزو/آي إي سي 42001: A.7.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.11; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
       </c>
       <c r="F26" t="str">
         <v>تم التحقق</v>
@@ -1245,25 +1245,25 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>CTL-HUM-03</v>
+        <v>CTL-DAT-05</v>
       </c>
       <c r="B27" t="str">
-        <v>الإشراف البشري</v>
+        <v>البيانات</v>
       </c>
       <c r="C27" t="str">
-        <v>الحدّ من الاعتماد المفرط على النظام</v>
+        <v>اختبار التحيّز والإنصاف</v>
       </c>
       <c r="D27" t="str">
-        <v>تدريب المراجعين على التحقق من مخرجات الذكاء الاصطناعي بدلًا من اعتمادها تلقائيًا، ومتابعة معدل تجاوزهم لتوصيات النظام بشكل دوري.</v>
+        <v>اختبار النتائج عبر الفئات ذات الصلة قبل الإطلاق وبعد التغييرات الجوهرية، مع تحديد حدّ مقبول مسبقًا، وتوثيق النتائج وأي إجراءات معالجة.</v>
       </c>
       <c r="E27" t="str">
-        <v>آيزو/آي إي سي 42001: A.4.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.4, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Algorithmic bias; أخلاقيات الذكاء الاصطناعي في دبي: Fairness; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Fairness; آيزو/آي إي سي 42001: A.5.4, A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.11; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
       </c>
       <c r="F27" t="str">
-        <v>تم التحقق</v>
+        <v>بحاجة إلى تحقق</v>
       </c>
       <c r="G27" t="str">
-        <v>مخاطر مرتفعة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -1277,25 +1277,25 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>CTL-HUM-04</v>
+        <v>CTL-DAT-06</v>
       </c>
       <c r="B28" t="str">
-        <v>الإشراف البشري</v>
+        <v>البيانات</v>
       </c>
       <c r="C28" t="str">
-        <v>حدود الاستقلالية للوكلاء الأذكياء</v>
+        <v>ضوابط إدخال البيانات في أدوات الذكاء الاصطناعي التوليدي</v>
       </c>
       <c r="D28" t="str">
-        <v>توثيق ما يُسمح للوكيل الذكي بفعله باستقلالية وما يُحظر عليه تمامًا، والحدود التي يعمل ضمنها (مثل المبالغ أو أنواع السجلات أو عدد الإجراءات)، وفرض هذه الحدود تقنيًا.</v>
+        <v>وضع قواعد واضحة لنوع المعلومات التي يجوز للموظفين إدخالها في أدوات الذكاء الاصطناعي التوليدي، ومنع إدخال البيانات الشخصية أو الحساسة أو المصنّفة في الخدمات الخارجية إلا بموافقة صريحة.</v>
       </c>
       <c r="E28" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.9.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.3, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.2.3, A.9.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MEASURE 2.10</v>
       </c>
       <c r="F28" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G28" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -1309,22 +1309,22 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>CTL-HUM-05</v>
+        <v>CTL-DAT-07</v>
       </c>
       <c r="B29" t="str">
-        <v>الإشراف البشري</v>
+        <v>البيانات</v>
       </c>
       <c r="C29" t="str">
-        <v>موافقة بشرية على الإجراءات غير القابلة للتراجع</v>
+        <v>حقوق استخدام محتوى التدريب والإسناد</v>
       </c>
       <c r="D29" t="str">
-        <v>اشتراط موافقة شخص محدد على أي إجراء يقوم به الوكيل الذكي ويصعب التراجع عنه أو يؤثر تأثيرًا مهمًا في الأفراد، مثل المدفوعات أو الحذف أو المراسلات الخارجية أو القرارات المتعلقة بالاستحقاقات.</v>
+        <v>التأكد من امتلاك الجهة حق استخدام الوثائق والمحتوى المستخدم في تدريب النموذج أو ضبطه أو إسناد إجاباته، والاحتفاظ بسجل لهذا التحقق.</v>
       </c>
       <c r="E29" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Human oversight; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.1.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.5, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
+        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.7.3, A.7.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 4.1, GOVERN 6.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 53</v>
       </c>
       <c r="F29" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G29" t="str">
         <v>مخاطر محدودة</v>
@@ -1341,19 +1341,19 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>CTL-HUM-06</v>
+        <v>CTL-DAT-08</v>
       </c>
       <c r="B30" t="str">
-        <v>الإشراف البشري</v>
+        <v>البيانات</v>
       </c>
       <c r="C30" t="str">
-        <v>آلية الإيقاف والتراجع</v>
+        <v>الاعتماد على المصادر الذهبية دون نسخ موازية</v>
       </c>
       <c r="D30" t="str">
-        <v>توفير آلية مُختبرة تمكّن الموظفين المخوّلين من إيقاف الوكيل الذكي مؤقتًا أو تعطيله فورًا، ومن عكس الإجراءات التي نفّذها أو تصحيحها.</v>
+        <v>أن تستقي أنظمة الذكاء الاصطناعي البيانات الحكومية من مصادرها الذهبية المعتمدة عند الحاجة إليها، وأن تستخدمها للغرض المصرّح به فقط، دون الاحتفاظ بنسخ منها لإعادة استخدامها أو بناء قواعد بيانات موازية.</v>
       </c>
       <c r="E30" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.3, Code 5.7, Data Sharing Policy Art. 5, Data Sharing Policy Art. 8</v>
       </c>
       <c r="F30" t="str">
         <v>تم التحقق</v>
@@ -1373,22 +1373,22 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>CTL-SEC-01</v>
+        <v>CTL-DAT-09</v>
       </c>
       <c r="B31" t="str">
-        <v>السلامة والأمن</v>
+        <v>البيانات</v>
       </c>
       <c r="C31" t="str">
-        <v>الاختبار قبل التشغيل</v>
+        <v>طلب البيانات مرة واحدة</v>
       </c>
       <c r="D31" t="str">
-        <v>اختبار النظام وفق معايير محددة للدقة والسلامة، بما في ذلك المدخلات غير المعتادة والحالات القصوى، وفي ظروف قريبة من الاستخدام الفعلي قبل تشغيله.</v>
+        <v>تصميم الخدمات التي يقدّمها الذكاء الاصطناعي بحيث لا تطلب من المتعامل أي بيانات أو مستندات متوفرة لدى الحكومة ومصرّح باستخدامها، بل تسترجعها من مصدرها، ولا تطلب إلا ما هو ناقص فعلًا مع توضيح سبب الحاجة إليه.</v>
       </c>
       <c r="E31" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Safety; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.5, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 1.5, Code 5.4, Agentic Guide §03, Agentic Guide §06, Data Sharing Policy Art. 5, Data Sharing Policy Art. 8</v>
       </c>
       <c r="F31" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G31" t="str">
         <v>مخاطر محدودة</v>
@@ -1405,22 +1405,22 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>CTL-SEC-02</v>
+        <v>CTL-HUM-01</v>
       </c>
       <c r="B32" t="str">
-        <v>السلامة والأمن</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C32" t="str">
-        <v>تقييم أمني خاص بالذكاء الاصطناعي</v>
+        <v>نموذج محدد للإشراف البشري</v>
       </c>
       <c r="D32" t="str">
-        <v>تقييم التهديدات الخاصة بالذكاء الاصطناعي مثل حقن الأوامر وتسميم البيانات وتسرّب البيانات عبر المخرجات، وتضمين المتطلبات الناتجة في مواصفات النظام.</v>
+        <v>تحديد وتوثيق مواضع مراجعة البشر لمخرجات النظام أو الموافقة عليها أو مراقبتها لكل حالة استخدام، وإسناد هذا الدور إلى أشخاص يملكون الكفاءة والصلاحية للتدخل.</v>
       </c>
       <c r="E32" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Human oversight; كود الإمارات للخدمات الحكومية: Code 5.4, Agentic Guide §05, Agentic Reference p.7; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.1.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.5, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14, Art. 26</v>
       </c>
       <c r="F32" t="str">
-        <v>تم التحقق</v>
+        <v>بحاجة إلى تحقق</v>
       </c>
       <c r="G32" t="str">
         <v>مخاطر محدودة</v>
@@ -1437,19 +1437,19 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>CTL-SEC-03</v>
+        <v>CTL-HUM-02</v>
       </c>
       <c r="B33" t="str">
-        <v>السلامة والأمن</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C33" t="str">
-        <v>ضوابط على المخرجات المُولَّدة</v>
+        <v>حق الاعتراض على القرار</v>
       </c>
       <c r="D33" t="str">
-        <v>وضع ضوابط على مخرجات الذكاء الاصطناعي التوليدي (الإسناد إلى مصادر معتمدة، وتصفية المحتوى الضار أو غير الصحيح، والمراجعة البشرية عند الحاجة) قبل وصولها إلى المتعاملين أو استخدامها في القرارات.</v>
+        <v>إتاحة مسار واضح للأفراد للاعتراض على أي قرار مهم استند إلى الذكاء الاصطناعي، ومراجعته من قِبل شخص مخوّل بتعديله.</v>
       </c>
       <c r="E33" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.6</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.4, Agentic Guide §03, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 3.3</v>
       </c>
       <c r="F33" t="str">
         <v>تم التحقق</v>
@@ -1469,25 +1469,25 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>CTL-SEC-04</v>
+        <v>CTL-HUM-03</v>
       </c>
       <c r="B34" t="str">
-        <v>السلامة والأمن</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C34" t="str">
-        <v>أقل صلاحيات ممكنة للأدوات والأذونات</v>
+        <v>الحدّ من الاعتماد المفرط على النظام</v>
       </c>
       <c r="D34" t="str">
-        <v>منح الوكيل الذكي صلاحية الوصول فقط إلى الأدوات والأنظمة والبيانات اللازمة لمهمته، مع جعل الوصول للقراءة فقط افتراضيًا ومنح صلاحية الكتابة لكل حالة على حدة.</v>
+        <v>تدريب المراجعين على التحقق من مخرجات الذكاء الاصطناعي بدلًا من اعتمادها تلقائيًا، ومتابعة معدل تجاوزهم لتوصيات النظام بشكل دوري.</v>
       </c>
       <c r="E34" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 4.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>آيزو/آي إي سي 42001: A.4.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.4, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
       </c>
       <c r="F34" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G34" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر مرتفعة</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -1501,19 +1501,19 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>CTL-SEC-05</v>
+        <v>CTL-HUM-04</v>
       </c>
       <c r="B35" t="str">
-        <v>السلامة والأمن</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C35" t="str">
-        <v>بيئة تجريبية وإطلاق تدريجي للوكلاء</v>
+        <v>حدود الاستقلالية للوكلاء الأذكياء</v>
       </c>
       <c r="D35" t="str">
-        <v>تشغيل الوكيل الذكي الجديد في بيئة اختبار أو وضع مراقبة تُسجَّل فيه الإجراءات المقترحة دون تنفيذها، قبل منحه وصولًا فعليًا، ثم توسيع نطاقه على مراحل.</v>
+        <v>توثيق ما يُسمح للوكيل الذكي بفعله باستقلالية وما يُحظر عليه تمامًا، والحدود التي يعمل ضمنها (مثل المبالغ أو أنواع السجلات أو عدد الإجراءات)، وفرض هذه الحدود تقنيًا.</v>
       </c>
       <c r="E35" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4, A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.3, MEASURE 2.6</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.4, Agentic Guide §05, Agentic Reference p.8; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.9.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.3, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
       </c>
       <c r="F35" t="str">
         <v>تم التحقق</v>
@@ -1533,22 +1533,22 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>CTL-SEC-06</v>
+        <v>CTL-HUM-05</v>
       </c>
       <c r="B36" t="str">
-        <v>السلامة والأمن</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C36" t="str">
-        <v>البديل الاحتياطي والتوقف الآمن</v>
+        <v>موافقة بشرية على الإجراءات غير القابلة للتراجع</v>
       </c>
       <c r="D36" t="str">
-        <v>تحديد ما يحدث عند تعطل النظام أو إيقافه، بما في ذلك وجود بديل يدوي أو غير معتمد على الذكاء الاصطناعي، لضمان استمرار الخدمة بأمان.</v>
+        <v>اشتراط موافقة شخص محدد على أي إجراء يقوم به الوكيل الذكي ويصعب التراجع عنه أو يؤثر تأثيرًا مهمًا في الأفراد، مثل المدفوعات أو الحذف أو المراسلات الخارجية أو القرارات المتعلقة بالاستحقاقات.</v>
       </c>
       <c r="E36" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 2.1, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Human oversight; كود الإمارات للخدمات الحكومية: Code 5.2, Agentic Guide §03; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.1.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.5, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
       </c>
       <c r="F36" t="str">
-        <v>تم التحقق</v>
+        <v>بحاجة إلى تحقق</v>
       </c>
       <c r="G36" t="str">
         <v>مخاطر محدودة</v>
@@ -1565,25 +1565,25 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>CTL-SEC-07</v>
+        <v>CTL-HUM-06</v>
       </c>
       <c r="B37" t="str">
-        <v>السلامة والأمن</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C37" t="str">
-        <v>فحص الاستخدامات المحظورة</v>
+        <v>آلية الإيقاف والتراجع</v>
       </c>
       <c r="D37" t="str">
-        <v>فحص كل حالة استخدام مقترحة للتأكد من عدم وقوعها ضمن الممارسات المحظورة، مثل التصنيف الاجتماعي أو التلاعب بالسلوك، وإيقاف أي حالة تندرج ضمنها.</v>
+        <v>توفير آلية مُختبرة تمكّن الموظفين المخوّلين من إيقاف الوكيل الذكي مؤقتًا أو تعطيله فورًا، ومن عكس الإجراءات التي نفّذها أو تصحيحها.</v>
       </c>
       <c r="E37" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.9.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 1.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 5</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.5; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
       </c>
       <c r="F37" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G37" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -1597,19 +1597,19 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>CTL-MON-01</v>
+        <v>CTL-HUM-07</v>
       </c>
       <c r="B38" t="str">
-        <v>المراقبة</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C38" t="str">
-        <v>مراقبة الأداء مع التنبيهات</v>
+        <v>موافقة محددة لكل إجراء ينفذه الوكيل</v>
       </c>
       <c r="D38" t="str">
-        <v>مراقبة أداء النظام أثناء التشغيل وفق مؤشرات متفق عليها، وتحديد حدود التنبيه مسبقًا، وإسناد كل تنبيه إلى شخص مسؤول عن الاستجابة له.</v>
+        <v>قبل أن ينفّذ الوكيل أي إجراء نيابةً عن المتعامل، يُعرض عليه مخطط مختصر وتُطلب موافقته على ذلك الإجراء بعينه وعلى البيانات التي سيستخدمها وأي تكلفة مترتبة، دون الاعتماد على تفويض عام مفتوح، مع توثيق كل موافقة أو رفض.</v>
       </c>
       <c r="E38" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 4.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26, Art. 72</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.2, Agentic Guide §03, Agentic Guide §06</v>
       </c>
       <c r="F38" t="str">
         <v>تم التحقق</v>
@@ -1629,19 +1629,19 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>CTL-MON-02</v>
+        <v>CTL-HUM-08</v>
       </c>
       <c r="B39" t="str">
-        <v>المراقبة</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C39" t="str">
-        <v>تسجيل الأحداث</v>
+        <v>سحب صلاحيات الوكيل بخطوة واحدة</v>
       </c>
       <c r="D39" t="str">
-        <v>تسجيل المدخلات والمخرجات وإصدار النموذج والأحداث الرئيسية تلقائيًا، والاحتفاظ بالسجلات مدة كافية للتحقيق في الشكاوى والحوادث.</v>
+        <v>تمكين المتعامل من إيقاف الوكيل أو سحب الصلاحيات والموافقات التي منحها له بخطوة واحدة، مع تطبيق السحب فورًا وإرسال تأكيد بذلك.</v>
       </c>
       <c r="E39" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12, Art. 26</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.2, Agentic Guide §02, Agentic Guide §06</v>
       </c>
       <c r="F39" t="str">
         <v>تم التحقق</v>
@@ -1661,25 +1661,25 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>CTL-MON-03</v>
+        <v>CTL-HUM-09</v>
       </c>
       <c r="B40" t="str">
-        <v>المراقبة</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C40" t="str">
-        <v>سجل تدقيق لإجراءات الوكيل</v>
+        <v>التحويل إلى موظف مع كامل السياق</v>
       </c>
       <c r="D40" t="str">
-        <v>تسجيل كل استدعاء لأداة وكل إجراء يقوم به الوكيل الذكي، مع المدخلات والمبرر والنتيجة وأي موافقة بشرية، في سجل لا يستطيع الوكيل نفسه تعديله.</v>
+        <v>تحويل الحالة إلى موظف عند طلب المتعامل، أو عندما تكون معقدة أو حساسة أو تتجاوز ما يُسمح للذكاء الاصطناعي بتنفيذه أو يتعذّر إكمالها، مع نقل الطلب والسياق والإجراءات المنفذة والموافقات حتى لا يضطر المتعامل إلى إعادة شرح حالته.</v>
       </c>
       <c r="E40" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 1.7, Code 8.2, Agentic Guide §03, Agentic Guide §06</v>
       </c>
       <c r="F40" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G40" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H40" t="str">
         <v/>
@@ -1693,25 +1693,25 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>CTL-MON-04</v>
+        <v>CTL-HUM-10</v>
       </c>
       <c r="B41" t="str">
-        <v>المراقبة</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C41" t="str">
-        <v>الاستجابة لحوادث الذكاء الاصطناعي</v>
+        <v>موافقة صريحة قبل أي عملية دفع</v>
       </c>
       <c r="D41" t="str">
-        <v>تحديد آلية الإبلاغ عن حوادث الذكاء الاصطناعي والأخطاء الجسيمة والتحقيق فيها ومعالجتها وإبلاغ المتأثرين بها، والجهات التنظيمية عند الاقتضاء.</v>
+        <v>قبل أن يُجري الوكيل أي عملية دفع، تُعرض الرسوم والبنود والمبلغ الإجمالي والجهة المستفيدة ووسيلة الدفع، وتؤخذ موافقة المتعامل الصريحة، ويتم الدفع عبر قنوات الدفع الحكومية المعتمدة فقط، مع متابعة أي مبلغ يُحصَّل دون إتمام الخدمة.</v>
       </c>
       <c r="E41" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 4.3, MANAGE 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 73</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 1.6, Code 5.8, Agentic Guide §03, Agentic Guide §06</v>
       </c>
       <c r="F41" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G41" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H41" t="str">
         <v/>
@@ -1725,22 +1725,22 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>CTL-MON-05</v>
+        <v>CTL-SEC-01</v>
       </c>
       <c r="B42" t="str">
-        <v>المراقبة</v>
+        <v>السلامة والأمن</v>
       </c>
       <c r="C42" t="str">
-        <v>المراجعة الدورية وإعادة تصنيف المخاطر</v>
+        <v>الاختبار قبل التشغيل</v>
       </c>
       <c r="D42" t="str">
-        <v>مراجعة كل نظام وفق جدول زمني محدد وبعد أي تغييرات جوهرية، والتحقق من انحراف الأداء والمخاطر المستجدة، وتحديث مستوى المخاطر والضوابط المطبّقة.</v>
+        <v>اختبار النظام وفق معايير محددة للدقة والسلامة، بما في ذلك المدخلات غير المعتادة والحالات القصوى، وفي ظروف قريبة من الاستخدام الفعلي قبل تشغيله.</v>
       </c>
       <c r="E42" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.5, MEASURE 3.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 9</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Safety; كود الإمارات للخدمات الحكومية: Code 8.8, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.5, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F42" t="str">
-        <v>تم التحقق</v>
+        <v>بحاجة إلى تحقق</v>
       </c>
       <c r="G42" t="str">
         <v>مخاطر محدودة</v>
@@ -1757,25 +1757,25 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>CTL-MON-06</v>
+        <v>CTL-SEC-02</v>
       </c>
       <c r="B43" t="str">
-        <v>المراقبة</v>
+        <v>السلامة والأمن</v>
       </c>
       <c r="C43" t="str">
-        <v>قناة للإبلاغ عن المخاوف</v>
+        <v>تقييم أمني خاص بالذكاء الاصطناعي</v>
       </c>
       <c r="D43" t="str">
-        <v>توفير قناة للموظفين والمستخدمين للإبلاغ عن المشكلات أو المخاوف المتعلقة بنظام الذكاء الاصطناعي، ومتابعة كل بلاغ حتى إغلاقه.</v>
+        <v>تقييم التهديدات الخاصة بالذكاء الاصطناعي مثل حقن الأوامر وتسميم البيانات وتسرّب البيانات عبر المخرجات، وتضمين المتطلبات الناتجة في مواصفات النظام.</v>
       </c>
       <c r="E43" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.3.3, A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 5.1, MEASURE 3.3</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F43" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G43" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -1789,25 +1789,25 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>CTL-MON-07</v>
+        <v>CTL-SEC-03</v>
       </c>
       <c r="B44" t="str">
-        <v>المراقبة</v>
+        <v>السلامة والأمن</v>
       </c>
       <c r="C44" t="str">
-        <v>الإيقاف النهائي الآمن</v>
+        <v>ضوابط على المخرجات المُولَّدة</v>
       </c>
       <c r="D44" t="str">
-        <v>وضع خطة لإيقاف النظام نهائيًا تشمل حذف البيانات أو أرشفتها وإلغاء صلاحيات الوصول وإبلاغ المستخدمين، والالتزام بها عند سحبه من الخدمة.</v>
+        <v>وضع ضوابط على مخرجات الذكاء الاصطناعي التوليدي (الإسناد إلى مصادر معتمدة، وتصفية المحتوى الضار أو غير الصحيح، والمراجعة البشرية عند الحاجة) قبل وصولها إلى المتعاملين أو استخدامها في القرارات.</v>
       </c>
       <c r="E44" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.7, MANAGE 2.4</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.6</v>
       </c>
       <c r="F44" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G44" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -1821,39 +1821,455 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
+        <v>CTL-SEC-04</v>
+      </c>
+      <c r="B45" t="str">
+        <v>السلامة والأمن</v>
+      </c>
+      <c r="C45" t="str">
+        <v>أقل صلاحيات ممكنة للأدوات والأذونات</v>
+      </c>
+      <c r="D45" t="str">
+        <v>منح الوكيل الذكي صلاحية الوصول فقط إلى الأدوات والأنظمة والبيانات اللازمة لمهمته، مع جعل الوصول للقراءة فقط افتراضيًا ومنح صلاحية الكتابة لكل حالة على حدة.</v>
+      </c>
+      <c r="E45" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 5.1, Code 5.7; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 4.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+      </c>
+      <c r="F45" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G45" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>CTL-SEC-05</v>
+      </c>
+      <c r="B46" t="str">
+        <v>السلامة والأمن</v>
+      </c>
+      <c r="C46" t="str">
+        <v>بيئة تجريبية وإطلاق تدريجي للوكلاء</v>
+      </c>
+      <c r="D46" t="str">
+        <v>تشغيل الوكيل الذكي الجديد في بيئة اختبار أو وضع مراقبة تُسجَّل فيه الإجراءات المقترحة دون تنفيذها، قبل منحه وصولًا فعليًا، ثم توسيع نطاقه على مراحل.</v>
+      </c>
+      <c r="E46" t="str">
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4, A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.3, MEASURE 2.6</v>
+      </c>
+      <c r="F46" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G46" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H46" t="str">
+        <v/>
+      </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>CTL-SEC-06</v>
+      </c>
+      <c r="B47" t="str">
+        <v>السلامة والأمن</v>
+      </c>
+      <c r="C47" t="str">
+        <v>البديل الاحتياطي والتوقف الآمن</v>
+      </c>
+      <c r="D47" t="str">
+        <v>تحديد ما يحدث عند تعطل النظام أو إيقافه، بما في ذلك وجود بديل يدوي أو غير معتمد على الذكاء الاصطناعي، لضمان استمرار الخدمة بأمان.</v>
+      </c>
+      <c r="E47" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 8.2; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 2.1, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+      </c>
+      <c r="F47" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G47" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>CTL-SEC-07</v>
+      </c>
+      <c r="B48" t="str">
+        <v>السلامة والأمن</v>
+      </c>
+      <c r="C48" t="str">
+        <v>فحص الاستخدامات المحظورة</v>
+      </c>
+      <c r="D48" t="str">
+        <v>فحص كل حالة استخدام مقترحة للتأكد من عدم وقوعها ضمن الممارسات المحظورة، مثل التصنيف الاجتماعي أو التلاعب بالسلوك، وإيقاف أي حالة تندرج ضمنها.</v>
+      </c>
+      <c r="E48" t="str">
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.9.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 1.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 5</v>
+      </c>
+      <c r="F48" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G48" t="str">
+        <v>مخاطر منخفضة أو معدومة</v>
+      </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>CTL-SEC-08</v>
+      </c>
+      <c r="B49" t="str">
+        <v>السلامة والأمن</v>
+      </c>
+      <c r="C49" t="str">
+        <v>التحقق من الهوية والصلاحية قبل كل إجراء مؤتمت</v>
+      </c>
+      <c r="D49" t="str">
+        <v>قبل أن ينفّذ الوكيل أو أي عملية مؤتمتة إجراءً ما، يجري التحقق من هوية الشخص الذي يعمل نيابةً عنه والتأكد من أن الإجراء يقع ضمن الصلاحيات المعتمدة، ويُمنع تنفيذه خلاف ذلك.</v>
+      </c>
+      <c r="E49" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 5.1; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security</v>
+      </c>
+      <c r="F49" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G49" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>CTL-MON-01</v>
+      </c>
+      <c r="B50" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C50" t="str">
+        <v>مراقبة الأداء مع التنبيهات</v>
+      </c>
+      <c r="D50" t="str">
+        <v>مراقبة أداء النظام أثناء التشغيل وفق مؤشرات متفق عليها، وتحديد حدود التنبيه مسبقًا، وإسناد كل تنبيه إلى شخص مسؤول عن الاستجابة له.</v>
+      </c>
+      <c r="E50" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 4.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26, Art. 72</v>
+      </c>
+      <c r="F50" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G50" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>CTL-MON-02</v>
+      </c>
+      <c r="B51" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C51" t="str">
+        <v>تسجيل الأحداث</v>
+      </c>
+      <c r="D51" t="str">
+        <v>تسجيل المدخلات والمخرجات وإصدار النموذج والأحداث الرئيسية تلقائيًا، والاحتفاظ بالسجلات مدة كافية للتحقيق في الشكاوى والحوادث.</v>
+      </c>
+      <c r="E51" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12, Art. 26</v>
+      </c>
+      <c r="F51" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G51" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>CTL-MON-03</v>
+      </c>
+      <c r="B52" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C52" t="str">
+        <v>سجل تدقيق لإجراءات الوكيل</v>
+      </c>
+      <c r="D52" t="str">
+        <v>تسجيل كل استدعاء لأداة وكل إجراء يقوم به الوكيل الذكي، مع المدخلات والمبرر والنتيجة وأي موافقة بشرية، في سجل لا يستطيع الوكيل نفسه تعديله.</v>
+      </c>
+      <c r="E52" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6, Agentic Guide §06, Agentic Reference p.9; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12</v>
+      </c>
+      <c r="F52" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G52" t="str">
+        <v>مخاطر منخفضة أو معدومة</v>
+      </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>CTL-MON-04</v>
+      </c>
+      <c r="B53" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C53" t="str">
+        <v>الاستجابة لحوادث الذكاء الاصطناعي</v>
+      </c>
+      <c r="D53" t="str">
+        <v>تحديد آلية الإبلاغ عن حوادث الذكاء الاصطناعي والأخطاء الجسيمة والتحقيق فيها ومعالجتها وإبلاغ المتأثرين بها، والجهات التنظيمية عند الاقتضاء.</v>
+      </c>
+      <c r="E53" t="str">
+        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 4.3, MANAGE 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 73</v>
+      </c>
+      <c r="F53" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G53" t="str">
+        <v>مخاطر منخفضة أو معدومة</v>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>CTL-MON-05</v>
+      </c>
+      <c r="B54" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C54" t="str">
+        <v>المراجعة الدورية وإعادة تصنيف المخاطر</v>
+      </c>
+      <c r="D54" t="str">
+        <v>مراجعة كل نظام وفق جدول زمني محدد وبعد أي تغييرات جوهرية، والتحقق من انحراف الأداء والمخاطر المستجدة، وتحديث مستوى المخاطر والضوابط المطبّقة.</v>
+      </c>
+      <c r="E54" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.5, MEASURE 3.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 9</v>
+      </c>
+      <c r="F54" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G54" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>CTL-MON-06</v>
+      </c>
+      <c r="B55" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C55" t="str">
+        <v>قناة للإبلاغ عن المخاوف</v>
+      </c>
+      <c r="D55" t="str">
+        <v>توفير قناة للموظفين والمستخدمين للإبلاغ عن المشكلات أو المخاوف المتعلقة بنظام الذكاء الاصطناعي، ومتابعة كل بلاغ حتى إغلاقه.</v>
+      </c>
+      <c r="E55" t="str">
+        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.3.3, A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 5.1, MEASURE 3.3</v>
+      </c>
+      <c r="F55" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G55" t="str">
+        <v>مخاطر منخفضة أو معدومة</v>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>CTL-MON-07</v>
+      </c>
+      <c r="B56" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C56" t="str">
+        <v>الإيقاف النهائي الآمن</v>
+      </c>
+      <c r="D56" t="str">
+        <v>وضع خطة لإيقاف النظام نهائيًا تشمل حذف البيانات أو أرشفتها وإلغاء صلاحيات الوصول وإبلاغ المستخدمين، والالتزام بها عند سحبه من الخدمة.</v>
+      </c>
+      <c r="E56" t="str">
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.7, MANAGE 2.4</v>
+      </c>
+      <c r="F56" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G56" t="str">
+        <v>مخاطر منخفضة أو معدومة</v>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
         <v>CTL-MON-08</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B57" t="str">
         <v>المراقبة</v>
       </c>
-      <c r="C45" t="str">
+      <c r="C57" t="str">
         <v>مراقبة سلوك الوكيل والإيقاف التلقائي</v>
       </c>
-      <c r="D45" t="str">
+      <c r="D57" t="str">
         <v>مراقبة الوكلاء الأذكياء لرصد السلوك غير المعتاد مثل التكرار المستمر أو الارتفاع المفاجئ في عدد الإجراءات أو التكلفة أو محاولة استخدام أدوات خارج نطاقهم، وإيقافهم تلقائيًا عند بلوغ الحدود.</v>
       </c>
-      <c r="E45" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 2.4</v>
-      </c>
-      <c r="F45" t="str">
-        <v>تم التحقق</v>
-      </c>
-      <c r="G45" t="str">
-        <v>مخاطر محدودة</v>
-      </c>
-      <c r="H45" t="str">
-        <v/>
-      </c>
-      <c r="I45" t="str">
-        <v/>
-      </c>
-      <c r="J45" t="str">
+      <c r="E57" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 5.5, Agentic Reference p.8; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 2.4</v>
+      </c>
+      <c r="F57" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G57" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>CTL-MON-09</v>
+      </c>
+      <c r="B58" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C58" t="str">
+        <v>مؤشرات أداء لكل وكيل وقرار الاستمرار أو الإيقاف</v>
+      </c>
+      <c r="D58" t="str">
+        <v>تحديد مؤشرات أداء لكل وكيل تشمل جودة القرارات والانحياز والأثر على الخدمة مقارنةً بخط أساس يُحدَّد قبل الإطلاق، ومراجعتها دوريًا مع مؤشرات رضا المتعاملين، وتوثيق قرار الاستمرار أو التعديل أو الإيقاف.</v>
+      </c>
+      <c r="E58" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1, Code 2.3, Agentic Guide §05, Agentic Guide §06; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 1.1</v>
+      </c>
+      <c r="F58" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G58" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(controls): add red-team testing and model supply chain security controls
A tester asked for explicit red-team and jailbreak testing and for model
supply-chain risk. CTL-SEC-02 stays the AI threat assessment. Two new
controls are split out of it:
- CTL-SEC-09, red-team and jailbreak testing, for generative and agentic
  AI from Limited, including indirect prompt injection through content the
  system reads;
- CTL-SEC-10, model supply chain security, for all AI types from Limited:
  inventory, trusted sources, integrity checks, pinned versions and
  vulnerability tracking.

Every reference was checked on 28 Sep 2026 against NIST AI 100-1, the
NIST-hosted ISO/IEC 42001 crosswalk and the Official Journal text of the
EU AI Act, and both rows are verified. CTL-SEC-02 also gains NIST MAP 1.6, the
crosswalk route to its ISO/IEC 42001 A.6.2.2 reference. Totals are now 58 controls, 50
verified. The content audit, README and templates are updated. See ADR 010.
</commit_message>
<xml_diff>
--- a/public/templates/ar/control-checklist.xlsx
+++ b/public/templates/ar/control-checklist.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J60"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1769,7 +1769,7 @@
         <v>تقييم التهديدات الخاصة بالذكاء الاصطناعي مثل حقن الأوامر وتسميم البيانات وتسرّب البيانات عبر المخرجات، وتضمين المتطلبات الناتجة في مواصفات النظام.</v>
       </c>
       <c r="E43" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 1.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F43" t="str">
         <v>تم التحقق</v>
@@ -1981,19 +1981,19 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>CTL-MON-01</v>
+        <v>CTL-SEC-09</v>
       </c>
       <c r="B50" t="str">
-        <v>المراقبة</v>
+        <v>السلامة والأمن</v>
       </c>
       <c r="C50" t="str">
-        <v>مراقبة الأداء مع التنبيهات</v>
+        <v>اختبار الفريق الأحمر ومحاولات كسر القيود</v>
       </c>
       <c r="D50" t="str">
-        <v>مراقبة أداء النظام أثناء التشغيل وفق مؤشرات متفق عليها، وتحديد حدود التنبيه مسبقًا، وإسناد كل تنبيه إلى شخص مسؤول عن الاستجابة له.</v>
+        <v>قبل الإطلاق وبعد كل تغيير جوهري، يُكلَّف أشخاص لم يشاركوا في بناء النظام بمحاولة دفعه إلى سلوك غير مقصود: محاولات كسر القيود، وحقن الأوامر المباشر وغير المباشر (بما في ذلك عبر المستندات أو الرسائل أو صفحات الويب التي يقرؤها)، واستخراج البيانات السرية، وإساءة استخدام أدواته. وتُوثَّق النتائج وتُعالَج ثم يُعاد الاختبار.</v>
       </c>
       <c r="E50" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 4.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26, Art. 72</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 1.3, MEASURE 2.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 55</v>
       </c>
       <c r="F50" t="str">
         <v>تم التحقق</v>
@@ -2013,19 +2013,19 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>CTL-MON-02</v>
+        <v>CTL-SEC-10</v>
       </c>
       <c r="B51" t="str">
-        <v>المراقبة</v>
+        <v>السلامة والأمن</v>
       </c>
       <c r="C51" t="str">
-        <v>تسجيل الأحداث</v>
+        <v>أمن سلسلة توريد النماذج</v>
       </c>
       <c r="D51" t="str">
-        <v>تسجيل المدخلات والمخرجات وإصدار النموذج والأحداث الرئيسية تلقائيًا، والاحتفاظ بالسجلات مدة كافية للتحقيق في الشكاوى والحوادث.</v>
+        <v>الاحتفاظ بقائمة بالنماذج ومجموعات البيانات ومكتبات الذكاء الاصطناعي التي يعتمد عليها النظام، مع مصدر كل منها وإصداره وترخيصه. وعدم الحصول عليها إلا من مصادر موثوقة، والتحقق من سلامتها قبل الاستخدام، وتثبيت إصداراتها، ومتابعة ثغراتها وتحديثاتها من المصدر، حتى لا يصل إلى بيئة التشغيل مكوّن جرى العبث به أو تحديثه دون علم.</v>
       </c>
       <c r="E51" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12, Art. 26</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.10.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MAP 4.1, MANAGE 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 25</v>
       </c>
       <c r="F51" t="str">
         <v>تم التحقق</v>
@@ -2045,25 +2045,25 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>CTL-MON-03</v>
+        <v>CTL-MON-01</v>
       </c>
       <c r="B52" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C52" t="str">
-        <v>سجل تدقيق لإجراءات الوكيل</v>
+        <v>مراقبة الأداء مع التنبيهات</v>
       </c>
       <c r="D52" t="str">
-        <v>تسجيل كل استدعاء لأداة وكل إجراء يقوم به الوكيل الذكي، مع المدخلات والمبرر والنتيجة وأي موافقة بشرية، في سجل لا يستطيع الوكيل نفسه تعديله.</v>
+        <v>مراقبة أداء النظام أثناء التشغيل وفق مؤشرات متفق عليها، وتحديد حدود التنبيه مسبقًا، وإسناد كل تنبيه إلى شخص مسؤول عن الاستجابة له.</v>
       </c>
       <c r="E52" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.6, Agentic Guide §06, Agentic Reference p.9; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 4.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26, Art. 72</v>
       </c>
       <c r="F52" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G52" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -2077,25 +2077,25 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>CTL-MON-04</v>
+        <v>CTL-MON-02</v>
       </c>
       <c r="B53" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C53" t="str">
-        <v>الاستجابة لحوادث الذكاء الاصطناعي</v>
+        <v>تسجيل الأحداث</v>
       </c>
       <c r="D53" t="str">
-        <v>تحديد آلية الإبلاغ عن حوادث الذكاء الاصطناعي والأخطاء الجسيمة والتحقيق فيها ومعالجتها وإبلاغ المتأثرين بها، والجهات التنظيمية عند الاقتضاء.</v>
+        <v>تسجيل المدخلات والمخرجات وإصدار النموذج والأحداث الرئيسية تلقائيًا، والاحتفاظ بالسجلات مدة كافية للتحقيق في الشكاوى والحوادث.</v>
       </c>
       <c r="E53" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 4.3, MANAGE 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 73</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12, Art. 26</v>
       </c>
       <c r="F53" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G53" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -2109,25 +2109,25 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>CTL-MON-05</v>
+        <v>CTL-MON-03</v>
       </c>
       <c r="B54" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C54" t="str">
-        <v>المراجعة الدورية وإعادة تصنيف المخاطر</v>
+        <v>سجل تدقيق لإجراءات الوكيل</v>
       </c>
       <c r="D54" t="str">
-        <v>مراجعة كل نظام وفق جدول زمني محدد وبعد أي تغييرات جوهرية، والتحقق من انحراف الأداء والمخاطر المستجدة، وتحديث مستوى المخاطر والضوابط المطبّقة.</v>
+        <v>تسجيل كل استدعاء لأداة وكل إجراء يقوم به الوكيل الذكي، مع المدخلات والمبرر والنتيجة وأي موافقة بشرية، في سجل لا يستطيع الوكيل نفسه تعديله.</v>
       </c>
       <c r="E54" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.5, MEASURE 3.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 9</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6, Agentic Guide §06, Agentic Reference p.9; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12</v>
       </c>
       <c r="F54" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G54" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -2141,19 +2141,19 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>CTL-MON-06</v>
+        <v>CTL-MON-04</v>
       </c>
       <c r="B55" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C55" t="str">
-        <v>قناة للإبلاغ عن المخاوف</v>
+        <v>الاستجابة لحوادث الذكاء الاصطناعي</v>
       </c>
       <c r="D55" t="str">
-        <v>توفير قناة للموظفين والمستخدمين للإبلاغ عن المشكلات أو المخاوف المتعلقة بنظام الذكاء الاصطناعي، ومتابعة كل بلاغ حتى إغلاقه.</v>
+        <v>تحديد آلية الإبلاغ عن حوادث الذكاء الاصطناعي والأخطاء الجسيمة والتحقيق فيها ومعالجتها وإبلاغ المتأثرين بها، والجهات التنظيمية عند الاقتضاء.</v>
       </c>
       <c r="E55" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.3.3, A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 5.1, MEASURE 3.3</v>
+        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 4.3, MANAGE 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 73</v>
       </c>
       <c r="F55" t="str">
         <v>تم التحقق</v>
@@ -2173,25 +2173,25 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>CTL-MON-07</v>
+        <v>CTL-MON-05</v>
       </c>
       <c r="B56" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C56" t="str">
-        <v>الإيقاف النهائي الآمن</v>
+        <v>المراجعة الدورية وإعادة تصنيف المخاطر</v>
       </c>
       <c r="D56" t="str">
-        <v>وضع خطة لإيقاف النظام نهائيًا تشمل حذف البيانات أو أرشفتها وإلغاء صلاحيات الوصول وإبلاغ المستخدمين، والالتزام بها عند سحبه من الخدمة.</v>
+        <v>مراجعة كل نظام وفق جدول زمني محدد وبعد أي تغييرات جوهرية، والتحقق من انحراف الأداء والمخاطر المستجدة، وتحديث مستوى المخاطر والضوابط المطبّقة.</v>
       </c>
       <c r="E56" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.7, MANAGE 2.4</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.5, MEASURE 3.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 9</v>
       </c>
       <c r="F56" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G56" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -2205,25 +2205,25 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>CTL-MON-08</v>
+        <v>CTL-MON-06</v>
       </c>
       <c r="B57" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C57" t="str">
-        <v>مراقبة سلوك الوكيل والإيقاف التلقائي</v>
+        <v>قناة للإبلاغ عن المخاوف</v>
       </c>
       <c r="D57" t="str">
-        <v>مراقبة الوكلاء الأذكياء لرصد السلوك غير المعتاد مثل التكرار المستمر أو الارتفاع المفاجئ في عدد الإجراءات أو التكلفة أو محاولة استخدام أدوات خارج نطاقهم، وإيقافهم تلقائيًا عند بلوغ الحدود.</v>
+        <v>توفير قناة للموظفين والمستخدمين للإبلاغ عن المشكلات أو المخاوف المتعلقة بنظام الذكاء الاصطناعي، ومتابعة كل بلاغ حتى إغلاقه.</v>
       </c>
       <c r="E57" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.5, Agentic Reference p.8; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 2.4</v>
+        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.3.3, A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 5.1, MEASURE 3.3</v>
       </c>
       <c r="F57" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G57" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -2237,39 +2237,103 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>CTL-MON-09</v>
+        <v>CTL-MON-07</v>
       </c>
       <c r="B58" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C58" t="str">
+        <v>الإيقاف النهائي الآمن</v>
+      </c>
+      <c r="D58" t="str">
+        <v>وضع خطة لإيقاف النظام نهائيًا تشمل حذف البيانات أو أرشفتها وإلغاء صلاحيات الوصول وإبلاغ المستخدمين، والالتزام بها عند سحبه من الخدمة.</v>
+      </c>
+      <c r="E58" t="str">
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.7, MANAGE 2.4</v>
+      </c>
+      <c r="F58" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G58" t="str">
+        <v>مخاطر منخفضة أو معدومة</v>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>CTL-MON-08</v>
+      </c>
+      <c r="B59" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C59" t="str">
+        <v>مراقبة سلوك الوكيل والإيقاف التلقائي</v>
+      </c>
+      <c r="D59" t="str">
+        <v>مراقبة الوكلاء الأذكياء لرصد السلوك غير المعتاد مثل التكرار المستمر أو الارتفاع المفاجئ في عدد الإجراءات أو التكلفة أو محاولة استخدام أدوات خارج نطاقهم، وإيقافهم تلقائيًا عند بلوغ الحدود.</v>
+      </c>
+      <c r="E59" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 5.5, Agentic Reference p.8; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 2.4</v>
+      </c>
+      <c r="F59" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G59" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
+      <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>CTL-MON-09</v>
+      </c>
+      <c r="B60" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C60" t="str">
         <v>مؤشرات أداء لكل وكيل وقرار الاستمرار أو الإيقاف</v>
       </c>
-      <c r="D58" t="str">
+      <c r="D60" t="str">
         <v>تحديد مؤشرات أداء لكل وكيل تشمل جودة القرارات والانحياز والأثر على الخدمة مقارنةً بخط أساس يُحدَّد قبل الإطلاق، ومراجعتها دوريًا مع مؤشرات رضا المتعاملين، وتوثيق قرار الاستمرار أو التعديل أو الإيقاف.</v>
       </c>
-      <c r="E58" t="str">
+      <c r="E60" t="str">
         <v>كود الإمارات للخدمات الحكومية: Code 2.1, Code 2.3, Agentic Guide §05, Agentic Guide §06; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 1.1</v>
       </c>
-      <c r="F58" t="str">
-        <v>تم التحقق</v>
-      </c>
-      <c r="G58" t="str">
-        <v>مخاطر محدودة</v>
-      </c>
-      <c r="H58" t="str">
-        <v/>
-      </c>
-      <c r="I58" t="str">
-        <v/>
-      </c>
-      <c r="J58" t="str">
+      <c r="F60" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G60" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+      <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J60"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(crosswalk): verify the 8 UAE AI Charter rows against the official text
The Charter pages block scripted fetches, so 8 rows shipped unverified in
v0.3.1. They were checked in a browser against the UAE Legislation portal
on 15 Oct 2026. Six names matched; the awareness principle is corrected to
'Promoting AI awareness for an inclusive future'. All 58 controls are now
verified. Adds tests that every row is verified and every Charter ref uses
an official principle name; regenerates the control-checklist templates.
</commit_message>
<xml_diff>
--- a/public/templates/ar/control-checklist.xlsx
+++ b/public/templates/ar/control-checklist.xlsx
@@ -524,7 +524,7 @@
         <v>ميثاق الإمارات للذكاء الاصطناعي: Governance and accountability; كود الإمارات للخدمات الحكومية: Agentic Reference p.9; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.3.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.1</v>
       </c>
       <c r="F4" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G4" t="str">
         <v>مخاطر منخفضة أو معدومة</v>
@@ -681,10 +681,10 @@
         <v>تدريب الموظفين الذين يطوّرون أنظمة الذكاء الاصطناعي أو يشغّلونها أو يعتمدون عليها على قدراتها وحدودها وعلى مسؤولياتهم، بما يتناسب مع أدوارهم.</v>
       </c>
       <c r="E9" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Promoting AI awareness for an inclusive society; كود الإمارات للخدمات الحكومية: Code 6.2; آيزو/آي إي سي 42001: A.4.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.2, MAP 3.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 4</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Promoting AI awareness for an inclusive future; كود الإمارات للخدمات الحكومية: Code 6.2; آيزو/آي إي سي 42001: A.4.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.2, MAP 3.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 4</v>
       </c>
       <c r="F9" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G9" t="str">
         <v>مخاطر منخفضة أو معدومة</v>
@@ -844,7 +844,7 @@
         <v>ميثاق الإمارات للذكاء الاصطناعي: Transparency; كود الإمارات للخدمات الحكومية: Code 5.6, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 50</v>
       </c>
       <c r="F14" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G14" t="str">
         <v>مخاطر منخفضة أو معدومة</v>
@@ -1196,7 +1196,7 @@
         <v>ميثاق الإمارات للذكاء الاصطناعي: Data privacy; كود الإمارات للخدمات الحكومية: Code 5.2, Code 5.7, Data Sharing Policy Art. 5; أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.2.3, A.7.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.10</v>
       </c>
       <c r="F25" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G25" t="str">
         <v>مخاطر منخفضة أو معدومة</v>
@@ -1260,7 +1260,7 @@
         <v>ميثاق الإمارات للذكاء الاصطناعي: Algorithmic bias; أخلاقيات الذكاء الاصطناعي في دبي: Fairness; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Fairness; آيزو/آي إي سي 42001: A.5.4, A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.11; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 10</v>
       </c>
       <c r="F27" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G27" t="str">
         <v>مخاطر محدودة</v>
@@ -1420,7 +1420,7 @@
         <v>ميثاق الإمارات للذكاء الاصطناعي: Human oversight; كود الإمارات للخدمات الحكومية: Code 5.4, Agentic Guide §05, Agentic Reference p.7; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.1.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.5, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14, Art. 26</v>
       </c>
       <c r="F32" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G32" t="str">
         <v>مخاطر محدودة</v>
@@ -1548,7 +1548,7 @@
         <v>ميثاق الإمارات للذكاء الاصطناعي: Human oversight; كود الإمارات للخدمات الحكومية: Code 5.2, Agentic Guide §03; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.1.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.5, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
       </c>
       <c r="F36" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G36" t="str">
         <v>مخاطر محدودة</v>
@@ -1740,7 +1740,7 @@
         <v>ميثاق الإمارات للذكاء الاصطناعي: Safety; كود الإمارات للخدمات الحكومية: Code 8.8, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.5, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F42" t="str">
-        <v>بحاجة إلى تحقق</v>
+        <v>تم التحقق</v>
       </c>
       <c r="G42" t="str">
         <v>مخاطر محدودة</v>

</xml_diff>

<commit_message>
feat(controls): add CTL-HUM-11 oversight effectiveness
Reviewers of the v0.4 proposals agreed that the commonest oversight
failure is a review that happens but catches nothing. CTL-HUM-11 asks
for evidence that review catches errors: known flawed cases in testing,
blind re-review of approved samples, evidence-based approval reasons,
reviewer volume caps, and approval-rate and review-time signals used as
triggers to investigate. See ADR 013. 59 controls, all verified.
</commit_message>
<xml_diff>
--- a/public/templates/ar/control-checklist.xlsx
+++ b/public/templates/ar/control-checklist.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J61"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1725,19 +1725,19 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>CTL-SEC-01</v>
+        <v>CTL-HUM-11</v>
       </c>
       <c r="B42" t="str">
-        <v>السلامة والأمن</v>
+        <v>الإشراف البشري</v>
       </c>
       <c r="C42" t="str">
-        <v>الاختبار قبل التشغيل</v>
+        <v>فاعلية الإشراف البشري</v>
       </c>
       <c r="D42" t="str">
-        <v>اختبار النظام وفق معايير محددة للدقة والسلامة، بما في ذلك المدخلات غير المعتادة والحالات القصوى، وفي ظروف قريبة من الاستخدام الفعلي قبل تشغيله.</v>
+        <v>إثبات أن المراجعة البشرية تكتشف الأخطاء فعلًا، لا أنها تتم شكليًا فقط: اختبار المراجعين بحالات معروفة الخطأ أثناء الاختبار أو التجربة، وإعادة مراجعة عينة من الحالات المعتمدة دون الاطلاع على القرار الأصلي، واشتراط أن يستند سبب الموافقة إلى دليل، ووضع حد أقصى لحجم العمل لكل مراجع، والتعامل مع معدلات الموافقة القريبة من 100% أو أوقات المراجعة القصيرة جدًا كمؤشرات تستدعي التحقق.</v>
       </c>
       <c r="E42" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Safety; كود الإمارات للخدمات الحكومية: Code 8.8, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.5, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Human oversight; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 3.5, GOVERN 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 14</v>
       </c>
       <c r="F42" t="str">
         <v>تم التحقق</v>
@@ -1757,19 +1757,19 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>CTL-SEC-02</v>
+        <v>CTL-SEC-01</v>
       </c>
       <c r="B43" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C43" t="str">
-        <v>تقييم أمني خاص بالذكاء الاصطناعي</v>
+        <v>الاختبار قبل التشغيل</v>
       </c>
       <c r="D43" t="str">
-        <v>تقييم التهديدات الخاصة بالذكاء الاصطناعي مثل حقن الأوامر وتسميم البيانات وتسرّب البيانات عبر المخرجات، وتضمين المتطلبات الناتجة في مواصفات النظام.</v>
+        <v>اختبار النظام وفق معايير محددة للدقة والسلامة، بما في ذلك المدخلات غير المعتادة والحالات القصوى، وفي ظروف قريبة من الاستخدام الفعلي قبل تشغيله.</v>
       </c>
       <c r="E43" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 1.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Safety; كود الإمارات للخدمات الحكومية: Code 8.8, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.5, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F43" t="str">
         <v>تم التحقق</v>
@@ -1789,19 +1789,19 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>CTL-SEC-03</v>
+        <v>CTL-SEC-02</v>
       </c>
       <c r="B44" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C44" t="str">
-        <v>ضوابط على المخرجات المُولَّدة</v>
+        <v>تقييم أمني خاص بالذكاء الاصطناعي</v>
       </c>
       <c r="D44" t="str">
-        <v>وضع ضوابط على مخرجات الذكاء الاصطناعي التوليدي (الإسناد إلى مصادر معتمدة، وتصفية المحتوى الضار أو غير الصحيح، والمراجعة البشرية عند الحاجة) قبل وصولها إلى المتعاملين أو استخدامها في القرارات.</v>
+        <v>تقييم التهديدات الخاصة بالذكاء الاصطناعي مثل حقن الأوامر وتسميم البيانات وتسرّب البيانات عبر المخرجات، وتضمين المتطلبات الناتجة في مواصفات النظام.</v>
       </c>
       <c r="E44" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.6</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 1.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F44" t="str">
         <v>تم التحقق</v>
@@ -1821,19 +1821,19 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>CTL-SEC-04</v>
+        <v>CTL-SEC-03</v>
       </c>
       <c r="B45" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C45" t="str">
-        <v>أقل صلاحيات ممكنة للأدوات والأذونات</v>
+        <v>ضوابط على المخرجات المُولَّدة</v>
       </c>
       <c r="D45" t="str">
-        <v>منح الوكيل الذكي صلاحية الوصول فقط إلى الأدوات والأنظمة والبيانات اللازمة لمهمته، مع جعل الوصول للقراءة فقط افتراضيًا ومنح صلاحية الكتابة لكل حالة على حدة.</v>
+        <v>وضع ضوابط على مخرجات الذكاء الاصطناعي التوليدي (الإسناد إلى مصادر معتمدة، وتصفية المحتوى الضار أو غير الصحيح، والمراجعة البشرية عند الحاجة) قبل وصولها إلى المتعاملين أو استخدامها في القرارات.</v>
       </c>
       <c r="E45" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.1, Code 5.7; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 4.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.6</v>
       </c>
       <c r="F45" t="str">
         <v>تم التحقق</v>
@@ -1853,19 +1853,19 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>CTL-SEC-05</v>
+        <v>CTL-SEC-04</v>
       </c>
       <c r="B46" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C46" t="str">
-        <v>بيئة تجريبية وإطلاق تدريجي للوكلاء</v>
+        <v>أقل صلاحيات ممكنة للأدوات والأذونات</v>
       </c>
       <c r="D46" t="str">
-        <v>تشغيل الوكيل الذكي الجديد في بيئة اختبار أو وضع مراقبة تُسجَّل فيه الإجراءات المقترحة دون تنفيذها، قبل منحه وصولًا فعليًا، ثم توسيع نطاقه على مراحل.</v>
+        <v>منح الوكيل الذكي صلاحية الوصول فقط إلى الأدوات والأنظمة والبيانات اللازمة لمهمته، مع جعل الوصول للقراءة فقط افتراضيًا ومنح صلاحية الكتابة لكل حالة على حدة.</v>
       </c>
       <c r="E46" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4, A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.3, MEASURE 2.6</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.1, Code 5.7; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 4.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F46" t="str">
         <v>تم التحقق</v>
@@ -1885,19 +1885,19 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>CTL-SEC-06</v>
+        <v>CTL-SEC-05</v>
       </c>
       <c r="B47" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C47" t="str">
-        <v>البديل الاحتياطي والتوقف الآمن</v>
+        <v>بيئة تجريبية وإطلاق تدريجي للوكلاء</v>
       </c>
       <c r="D47" t="str">
-        <v>تحديد ما يحدث عند تعطل النظام أو إيقافه، بما في ذلك وجود بديل يدوي أو غير معتمد على الذكاء الاصطناعي، لضمان استمرار الخدمة بأمان.</v>
+        <v>تشغيل الوكيل الذكي الجديد في بيئة اختبار أو وضع مراقبة تُسجَّل فيه الإجراءات المقترحة دون تنفيذها، قبل منحه وصولًا فعليًا، ثم توسيع نطاقه على مراحل.</v>
       </c>
       <c r="E47" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 8.2; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 2.1, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4, A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.3, MEASURE 2.6</v>
       </c>
       <c r="F47" t="str">
         <v>تم التحقق</v>
@@ -1917,25 +1917,25 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>CTL-SEC-07</v>
+        <v>CTL-SEC-06</v>
       </c>
       <c r="B48" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C48" t="str">
-        <v>فحص الاستخدامات المحظورة</v>
+        <v>البديل الاحتياطي والتوقف الآمن</v>
       </c>
       <c r="D48" t="str">
-        <v>فحص كل حالة استخدام مقترحة للتأكد من عدم وقوعها ضمن الممارسات المحظورة، مثل التصنيف الاجتماعي أو التلاعب بالسلوك، وإيقاف أي حالة تندرج ضمنها.</v>
+        <v>تحديد ما يحدث عند تعطل النظام أو إيقافه، بما في ذلك وجود بديل يدوي أو غير معتمد على الذكاء الاصطناعي، لضمان استمرار الخدمة بأمان.</v>
       </c>
       <c r="E48" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.9.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 1.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 5</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 8.2; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 2.1, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F48" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G48" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -1949,25 +1949,25 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>CTL-SEC-08</v>
+        <v>CTL-SEC-07</v>
       </c>
       <c r="B49" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C49" t="str">
-        <v>التحقق من الهوية والصلاحية قبل كل إجراء مؤتمت</v>
+        <v>فحص الاستخدامات المحظورة</v>
       </c>
       <c r="D49" t="str">
-        <v>قبل أن ينفّذ الوكيل أو أي عملية مؤتمتة إجراءً ما، يجري التحقق من هوية الشخص الذي يعمل نيابةً عنه والتأكد من أن الإجراء يقع ضمن الصلاحيات المعتمدة، ويُمنع تنفيذه خلاف ذلك.</v>
+        <v>فحص كل حالة استخدام مقترحة للتأكد من عدم وقوعها ضمن الممارسات المحظورة، مثل التصنيف الاجتماعي أو التلاعب بالسلوك، وإيقاف أي حالة تندرج ضمنها.</v>
       </c>
       <c r="E49" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.1; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.9.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 1.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 5</v>
       </c>
       <c r="F49" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G49" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H49" t="str">
         <v/>
@@ -1981,19 +1981,19 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>CTL-SEC-09</v>
+        <v>CTL-SEC-08</v>
       </c>
       <c r="B50" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C50" t="str">
-        <v>اختبار الفريق الأحمر ومحاولات كسر القيود</v>
+        <v>التحقق من الهوية والصلاحية قبل كل إجراء مؤتمت</v>
       </c>
       <c r="D50" t="str">
-        <v>قبل الإطلاق وبعد كل تغيير جوهري، يُكلَّف أشخاص لم يشاركوا في بناء النظام بمحاولة دفعه إلى سلوك غير مقصود: محاولات كسر القيود، وحقن الأوامر المباشر وغير المباشر (بما في ذلك عبر المستندات أو الرسائل أو صفحات الويب التي يقرؤها)، واستخراج البيانات السرية، وإساءة استخدام أدواته. وتُوثَّق النتائج وتُعالَج ثم يُعاد الاختبار.</v>
+        <v>قبل أن ينفّذ الوكيل أو أي عملية مؤتمتة إجراءً ما، يجري التحقق من هوية الشخص الذي يعمل نيابةً عنه والتأكد من أن الإجراء يقع ضمن الصلاحيات المعتمدة، ويُمنع تنفيذه خلاف ذلك.</v>
       </c>
       <c r="E50" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 1.3, MEASURE 2.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 55</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.1; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security</v>
       </c>
       <c r="F50" t="str">
         <v>تم التحقق</v>
@@ -2013,19 +2013,19 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>CTL-SEC-10</v>
+        <v>CTL-SEC-09</v>
       </c>
       <c r="B51" t="str">
         <v>السلامة والأمن</v>
       </c>
       <c r="C51" t="str">
-        <v>أمن سلسلة توريد النماذج</v>
+        <v>اختبار الفريق الأحمر ومحاولات كسر القيود</v>
       </c>
       <c r="D51" t="str">
-        <v>الاحتفاظ بقائمة بالنماذج ومجموعات البيانات ومكتبات الذكاء الاصطناعي التي يعتمد عليها النظام، مع مصدر كل منها وإصداره وترخيصه. وعدم الحصول عليها إلا من مصادر موثوقة، والتحقق من سلامتها قبل الاستخدام، وتثبيت إصداراتها، ومتابعة ثغراتها وتحديثاتها من المصدر، حتى لا يصل إلى بيئة التشغيل مكوّن جرى العبث به أو تحديثه دون علم.</v>
+        <v>قبل الإطلاق وبعد كل تغيير جوهري، يُكلَّف أشخاص لم يشاركوا في بناء النظام بمحاولة دفعه إلى سلوك غير مقصود: محاولات كسر القيود، وحقن الأوامر المباشر وغير المباشر (بما في ذلك عبر المستندات أو الرسائل أو صفحات الويب التي يقرؤها)، واستخراج البيانات السرية، وإساءة استخدام أدواته. وتُوثَّق النتائج وتُعالَج ثم يُعاد الاختبار.</v>
       </c>
       <c r="E51" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.10.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MAP 4.1, MANAGE 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 25</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 1.3, MEASURE 2.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 55</v>
       </c>
       <c r="F51" t="str">
         <v>تم التحقق</v>
@@ -2045,19 +2045,19 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>CTL-MON-01</v>
+        <v>CTL-SEC-10</v>
       </c>
       <c r="B52" t="str">
-        <v>المراقبة</v>
+        <v>السلامة والأمن</v>
       </c>
       <c r="C52" t="str">
-        <v>مراقبة الأداء مع التنبيهات</v>
+        <v>أمن سلسلة توريد النماذج</v>
       </c>
       <c r="D52" t="str">
-        <v>مراقبة أداء النظام أثناء التشغيل وفق مؤشرات متفق عليها، وتحديد حدود التنبيه مسبقًا، وإسناد كل تنبيه إلى شخص مسؤول عن الاستجابة له.</v>
+        <v>الاحتفاظ بقائمة بالنماذج ومجموعات البيانات ومكتبات الذكاء الاصطناعي التي يعتمد عليها النظام، مع مصدر كل منها وإصداره وترخيصه. وعدم الحصول عليها إلا من مصادر موثوقة، والتحقق من سلامتها قبل الاستخدام، وتثبيت إصداراتها، ومتابعة ثغراتها وتحديثاتها من المصدر، حتى لا يصل إلى بيئة التشغيل مكوّن جرى العبث به أو تحديثه دون علم.</v>
       </c>
       <c r="E52" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 4.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26, Art. 72</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.10.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MAP 4.1, MANAGE 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 25</v>
       </c>
       <c r="F52" t="str">
         <v>تم التحقق</v>
@@ -2077,19 +2077,19 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>CTL-MON-02</v>
+        <v>CTL-MON-01</v>
       </c>
       <c r="B53" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C53" t="str">
-        <v>تسجيل الأحداث</v>
+        <v>مراقبة الأداء مع التنبيهات</v>
       </c>
       <c r="D53" t="str">
-        <v>تسجيل المدخلات والمخرجات وإصدار النموذج والأحداث الرئيسية تلقائيًا، والاحتفاظ بالسجلات مدة كافية للتحقيق في الشكاوى والحوادث.</v>
+        <v>مراقبة أداء النظام أثناء التشغيل وفق مؤشرات متفق عليها، وتحديد حدود التنبيه مسبقًا، وإسناد كل تنبيه إلى شخص مسؤول عن الاستجابة له.</v>
       </c>
       <c r="E53" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12, Art. 26</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 4.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26, Art. 72</v>
       </c>
       <c r="F53" t="str">
         <v>تم التحقق</v>
@@ -2109,25 +2109,25 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>CTL-MON-03</v>
+        <v>CTL-MON-02</v>
       </c>
       <c r="B54" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C54" t="str">
-        <v>سجل تدقيق لإجراءات الوكيل</v>
+        <v>تسجيل الأحداث</v>
       </c>
       <c r="D54" t="str">
-        <v>تسجيل كل استدعاء لأداة وكل إجراء يقوم به الوكيل الذكي، مع المدخلات والمبرر والنتيجة وأي موافقة بشرية، في سجل لا يستطيع الوكيل نفسه تعديله.</v>
+        <v>تسجيل المدخلات والمخرجات وإصدار النموذج والأحداث الرئيسية تلقائيًا، والاحتفاظ بالسجلات مدة كافية للتحقيق في الشكاوى والحوادث.</v>
       </c>
       <c r="E54" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.6, Agentic Guide §06, Agentic Reference p.9; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12, Art. 26</v>
       </c>
       <c r="F54" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G54" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -2141,19 +2141,19 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>CTL-MON-04</v>
+        <v>CTL-MON-03</v>
       </c>
       <c r="B55" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C55" t="str">
-        <v>الاستجابة لحوادث الذكاء الاصطناعي</v>
+        <v>سجل تدقيق لإجراءات الوكيل</v>
       </c>
       <c r="D55" t="str">
-        <v>تحديد آلية الإبلاغ عن حوادث الذكاء الاصطناعي والأخطاء الجسيمة والتحقيق فيها ومعالجتها وإبلاغ المتأثرين بها، والجهات التنظيمية عند الاقتضاء.</v>
+        <v>تسجيل كل استدعاء لأداة وكل إجراء يقوم به الوكيل الذكي، مع المدخلات والمبرر والنتيجة وأي موافقة بشرية، في سجل لا يستطيع الوكيل نفسه تعديله.</v>
       </c>
       <c r="E55" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 4.3, MANAGE 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 73</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6, Agentic Guide §06, Agentic Reference p.9; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.6.2.8; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 12</v>
       </c>
       <c r="F55" t="str">
         <v>تم التحقق</v>
@@ -2173,25 +2173,25 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>CTL-MON-05</v>
+        <v>CTL-MON-04</v>
       </c>
       <c r="B56" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C56" t="str">
-        <v>المراجعة الدورية وإعادة تصنيف المخاطر</v>
+        <v>الاستجابة لحوادث الذكاء الاصطناعي</v>
       </c>
       <c r="D56" t="str">
-        <v>مراجعة كل نظام وفق جدول زمني محدد وبعد أي تغييرات جوهرية، والتحقق من انحراف الأداء والمخاطر المستجدة، وتحديث مستوى المخاطر والضوابط المطبّقة.</v>
+        <v>تحديد آلية الإبلاغ عن حوادث الذكاء الاصطناعي والأخطاء الجسيمة والتحقيق فيها ومعالجتها وإبلاغ المتأثرين بها، والجهات التنظيمية عند الاقتضاء.</v>
       </c>
       <c r="E56" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.5, MEASURE 3.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 9</v>
+        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 4.3, MANAGE 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 73</v>
       </c>
       <c r="F56" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G56" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -2205,25 +2205,25 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>CTL-MON-06</v>
+        <v>CTL-MON-05</v>
       </c>
       <c r="B57" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C57" t="str">
-        <v>قناة للإبلاغ عن المخاوف</v>
+        <v>المراجعة الدورية وإعادة تصنيف المخاطر</v>
       </c>
       <c r="D57" t="str">
-        <v>توفير قناة للموظفين والمستخدمين للإبلاغ عن المشكلات أو المخاوف المتعلقة بنظام الذكاء الاصطناعي، ومتابعة كل بلاغ حتى إغلاقه.</v>
+        <v>مراجعة كل نظام وفق جدول زمني محدد وبعد أي تغييرات جوهرية، والتحقق من انحراف الأداء والمخاطر المستجدة، وتحديث مستوى المخاطر والضوابط المطبّقة.</v>
       </c>
       <c r="E57" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.3.3, A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 5.1, MEASURE 3.3</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.5, MEASURE 3.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 9</v>
       </c>
       <c r="F57" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G57" t="str">
-        <v>مخاطر منخفضة أو معدومة</v>
+        <v>مخاطر محدودة</v>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -2237,19 +2237,19 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>CTL-MON-07</v>
+        <v>CTL-MON-06</v>
       </c>
       <c r="B58" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C58" t="str">
-        <v>الإيقاف النهائي الآمن</v>
+        <v>قناة للإبلاغ عن المخاوف</v>
       </c>
       <c r="D58" t="str">
-        <v>وضع خطة لإيقاف النظام نهائيًا تشمل حذف البيانات أو أرشفتها وإلغاء صلاحيات الوصول وإبلاغ المستخدمين، والالتزام بها عند سحبه من الخدمة.</v>
+        <v>توفير قناة للموظفين والمستخدمين للإبلاغ عن المشكلات أو المخاوف المتعلقة بنظام الذكاء الاصطناعي، ومتابعة كل بلاغ حتى إغلاقه.</v>
       </c>
       <c r="E58" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.7, MANAGE 2.4</v>
+        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.3.3, A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 5.1, MEASURE 3.3</v>
       </c>
       <c r="F58" t="str">
         <v>تم التحقق</v>
@@ -2269,25 +2269,25 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>CTL-MON-08</v>
+        <v>CTL-MON-07</v>
       </c>
       <c r="B59" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C59" t="str">
-        <v>مراقبة سلوك الوكيل والإيقاف التلقائي</v>
+        <v>الإيقاف النهائي الآمن</v>
       </c>
       <c r="D59" t="str">
-        <v>مراقبة الوكلاء الأذكياء لرصد السلوك غير المعتاد مثل التكرار المستمر أو الارتفاع المفاجئ في عدد الإجراءات أو التكلفة أو محاولة استخدام أدوات خارج نطاقهم، وإيقافهم تلقائيًا عند بلوغ الحدود.</v>
+        <v>وضع خطة لإيقاف النظام نهائيًا تشمل حذف البيانات أو أرشفتها وإلغاء صلاحيات الوصول وإبلاغ المستخدمين، والالتزام بها عند سحبه من الخدمة.</v>
       </c>
       <c r="E59" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.5, Agentic Reference p.8; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 2.4</v>
+        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.7, MANAGE 2.4</v>
       </c>
       <c r="F59" t="str">
         <v>تم التحقق</v>
       </c>
       <c r="G59" t="str">
-        <v>مخاطر محدودة</v>
+        <v>مخاطر منخفضة أو معدومة</v>
       </c>
       <c r="H59" t="str">
         <v/>
@@ -2301,39 +2301,71 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>CTL-MON-09</v>
+        <v>CTL-MON-08</v>
       </c>
       <c r="B60" t="str">
         <v>المراقبة</v>
       </c>
       <c r="C60" t="str">
+        <v>مراقبة سلوك الوكيل والإيقاف التلقائي</v>
+      </c>
+      <c r="D60" t="str">
+        <v>مراقبة الوكلاء الأذكياء لرصد السلوك غير المعتاد مثل التكرار المستمر أو الارتفاع المفاجئ في عدد الإجراءات أو التكلفة أو محاولة استخدام أدوات خارج نطاقهم، وإيقافهم تلقائيًا عند بلوغ الحدود.</v>
+      </c>
+      <c r="E60" t="str">
+        <v>كود الإمارات للخدمات الحكومية: Code 5.5, Agentic Reference p.8; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 2.4</v>
+      </c>
+      <c r="F60" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G60" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+      <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>CTL-MON-09</v>
+      </c>
+      <c r="B61" t="str">
+        <v>المراقبة</v>
+      </c>
+      <c r="C61" t="str">
         <v>مؤشرات أداء لكل وكيل وقرار الاستمرار أو الإيقاف</v>
       </c>
-      <c r="D60" t="str">
+      <c r="D61" t="str">
         <v>تحديد مؤشرات أداء لكل وكيل تشمل جودة القرارات والانحياز والأثر على الخدمة مقارنةً بخط أساس يُحدَّد قبل الإطلاق، ومراجعتها دوريًا مع مؤشرات رضا المتعاملين، وتوثيق قرار الاستمرار أو التعديل أو الإيقاف.</v>
       </c>
-      <c r="E60" t="str">
+      <c r="E61" t="str">
         <v>كود الإمارات للخدمات الحكومية: Code 2.1, Code 2.3, Agentic Guide §05, Agentic Guide §06; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 1.1</v>
       </c>
-      <c r="F60" t="str">
-        <v>تم التحقق</v>
-      </c>
-      <c r="G60" t="str">
-        <v>مخاطر محدودة</v>
-      </c>
-      <c r="H60" t="str">
-        <v/>
-      </c>
-      <c r="I60" t="str">
-        <v/>
-      </c>
-      <c r="J60" t="str">
+      <c r="F61" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="G61" t="str">
+        <v>مخاطر محدودة</v>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+      <c r="I61" t="str">
+        <v/>
+      </c>
+      <c r="J61" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(crosswalk): add UAE PDPL and the CSC AI Security Policy
Maps controls to two more UAE sources, suggested by the AI Safety UAE
community: the Personal Data Protection Law (Federal Decree-Law 45/2021;
8 controls, by article) and the Cyber Security Council's National Cyber
Security Policy for AI v1.1 (15 controls, by policy statement). Both were
read in full and every reference checked. The content audit explains PDPL's
carve-out for government entities and what was deliberately not mapped.
Adds both frameworks to the filters, reference links and templates.
</commit_message>
<xml_diff>
--- a/public/templates/ar/control-checklist.xlsx
+++ b/public/templates/ar/control-checklist.xlsx
@@ -489,7 +489,7 @@
         <v>اعتماد سياسة للذكاء الاصطناعي من الإدارة العليا تحدد مبادئ الجهة ومستوى المخاطر المقبول وقواعد الموافقة على الاستخدامات، مع مراجعتها سنويًا على الأقل.</v>
       </c>
       <c r="E3" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.2.2, A.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.2, GOVERN 2.3</v>
+        <v>السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.1.1; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.2.2, A.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.2, GOVERN 2.3</v>
       </c>
       <c r="F3" t="str">
         <v>تم التحقق</v>
@@ -553,7 +553,7 @@
         <v>الاحتفاظ بسجل موحّد لجميع أنظمة الذكاء الاصطناعي المستخدمة أو قيد التطوير، يتضمن المالك والغرض والبيانات المستخدمة ومستوى المخاطر والحالة، وتحديثه باستمرار.</v>
       </c>
       <c r="E5" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.4.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.6</v>
+        <v>السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.4.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 1.6</v>
       </c>
       <c r="F5" t="str">
         <v>تم التحقق</v>
@@ -585,7 +585,7 @@
         <v>إجراء تقييم للأثر المحتمل على الأفراد والفئات والجهة قبل الموافقة على حالة الاستخدام، وتوثيق النتائج، وإعادة التقييم عند حدوث تغيير جوهري في النظام.</v>
       </c>
       <c r="E6" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.5.2, A.5.3, A.5.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 1.1, MAP 5.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 9, Art. 27</v>
+        <v>قانون حماية البيانات الشخصية: Art. 21; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.1.2; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; آيزو/آي إي سي 42001: A.5.2, A.5.3, A.5.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 1.1, MAP 5.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 9, Art. 27</v>
       </c>
       <c r="F6" t="str">
         <v>تم التحقق</v>
@@ -649,7 +649,7 @@
         <v>قبل شراء نموذج أو خدمة ذكاء اصطناعي من طرف ثالث أو دمجها، يجب مراجعة توثيقها وطريقة معالجتها للبيانات وحدودها المعروفة، وتحديد مسؤوليات الإشراف والحوادث والتحديثات في العقد.</v>
       </c>
       <c r="E8" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.10.2, A.10.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MANAGE 3.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 25</v>
+        <v>قانون حماية البيانات الشخصية: Art. 8; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.1.3; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.10.2, A.10.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MANAGE 3.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 25</v>
       </c>
       <c r="F8" t="str">
         <v>تم التحقق</v>
@@ -681,7 +681,7 @@
         <v>تدريب الموظفين الذين يطوّرون أنظمة الذكاء الاصطناعي أو يشغّلونها أو يعتمدون عليها على قدراتها وحدودها وعلى مسؤولياتهم، بما يتناسب مع أدوارهم.</v>
       </c>
       <c r="E9" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Promoting AI awareness for an inclusive future; كود الإمارات للخدمات الحكومية: Code 6.2; آيزو/آي إي سي 42001: A.4.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.2, MAP 3.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 4</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Promoting AI awareness for an inclusive future; كود الإمارات للخدمات الحكومية: Code 6.2; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.5.1; آيزو/آي إي سي 42001: A.4.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 2.2, MAP 3.4; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 4</v>
       </c>
       <c r="F9" t="str">
         <v>تم التحقق</v>
@@ -905,7 +905,7 @@
         <v>توفير وسيلة ميسّرة تتيح للشخص المتأثر بقرار مهم استند إلى الذكاء الاصطناعي طلب تفسير بلغة واضحة للعوامل الرئيسية وراء القرار والحصول عليه.</v>
       </c>
       <c r="E16" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Explainability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.9; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 86</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6; قانون حماية البيانات الشخصية: Art. 13; أخلاقيات الذكاء الاصطناعي في دبي: Explainability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.9; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 86</v>
       </c>
       <c r="F16" t="str">
         <v>تم التحقق</v>
@@ -937,7 +937,7 @@
         <v>إخطار الأفراد عندما يُتخذ قرار يؤثر فيهم تأثيرًا مهمًا بواسطة نظام ذكاء اصطناعي أو بدعم منه، بمن فيهم الموظفون المتأثرون باستخدامه في بيئة العمل.</v>
       </c>
       <c r="E17" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 5.6; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.5; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 5.6; قانون حماية البيانات الشخصية: Art. 13; أخلاقيات الذكاء الاصطناعي في دبي: Transparency; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.5; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26</v>
       </c>
       <c r="F17" t="str">
         <v>تم التحقق</v>
@@ -1193,7 +1193,7 @@
         <v>عند استخدام بيانات شخصية، يجب إجراء مراجعة للخصوصية والاقتصار على الحد الأدنى من البيانات الشخصية اللازمة للغرض، بما يتوافق مع سياسة حماية البيانات في الجهة.</v>
       </c>
       <c r="E25" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Data privacy; كود الإمارات للخدمات الحكومية: Code 5.2, Code 5.7, Data Sharing Policy Art. 5; أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.2.3, A.7.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.10</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Data privacy; كود الإمارات للخدمات الحكومية: Code 5.2, Code 5.7, Data Sharing Policy Art. 5; قانون حماية البيانات الشخصية: Art. 5, Art. 21; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.3.5; أخلاقيات الذكاء الاصطناعي في دبي: Privacy; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.2.3, A.7.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.10</v>
       </c>
       <c r="F25" t="str">
         <v>تم التحقق</v>
@@ -1449,7 +1449,7 @@
         <v>إتاحة مسار واضح للأفراد للاعتراض على أي قرار مهم استند إلى الذكاء الاصطناعي، ومراجعته من قِبل شخص مخوّل بتعديله.</v>
       </c>
       <c r="E33" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 2.4, Agentic Guide §03, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 3.3</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.4, Agentic Guide §03, Agentic Guide §06; قانون حماية البيانات الشخصية: Art. 18; أخلاقيات الذكاء الاصطناعي في دبي: Accountability; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 3.3</v>
       </c>
       <c r="F33" t="str">
         <v>تم التحقق</v>
@@ -1769,7 +1769,7 @@
         <v>اختبار النظام وفق معايير محددة للدقة والسلامة، بما في ذلك المدخلات غير المعتادة والحالات القصوى، وفي ظروف قريبة من الاستخدام الفعلي قبل تشغيله.</v>
       </c>
       <c r="E43" t="str">
-        <v>ميثاق الإمارات للذكاء الاصطناعي: Safety; كود الإمارات للخدمات الحكومية: Code 8.8, Agentic Guide §06; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.5, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>ميثاق الإمارات للذكاء الاصطناعي: Safety; كود الإمارات للخدمات الحكومية: Code 8.8, Agentic Guide §06; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.4.4; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.5, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F43" t="str">
         <v>تم التحقق</v>
@@ -1801,7 +1801,7 @@
         <v>تقييم التهديدات الخاصة بالذكاء الاصطناعي مثل حقن الأوامر وتسميم البيانات وتسرّب البيانات عبر المخرجات، وتضمين المتطلبات الناتجة في مواصفات النظام.</v>
       </c>
       <c r="E44" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 1.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>قانون حماية البيانات الشخصية: Art. 20; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.1.2, 2.3.2; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.2; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MAP 1.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F44" t="str">
         <v>تم التحقق</v>
@@ -1833,7 +1833,7 @@
         <v>وضع ضوابط على مخرجات الذكاء الاصطناعي التوليدي (الإسناد إلى مصادر معتمدة، وتصفية المحتوى الضار أو غير الصحيح، والمراجعة البشرية عند الحاجة) قبل وصولها إلى المتعاملين أو استخدامها في القرارات.</v>
       </c>
       <c r="E45" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.6</v>
+        <v>السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.3.3; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.6</v>
       </c>
       <c r="F45" t="str">
         <v>تم التحقق</v>
@@ -1897,7 +1897,7 @@
         <v>تشغيل الوكيل الذكي الجديد في بيئة اختبار أو وضع مراقبة تُسجَّل فيه الإجراءات المقترحة دون تنفيذها، قبل منحه وصولًا فعليًا، ثم توسيع نطاقه على مراحل.</v>
       </c>
       <c r="E47" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4, A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.3, MEASURE 2.6</v>
+        <v>السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.1.4; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.4, A.6.2.5; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.3, MEASURE 2.6</v>
       </c>
       <c r="F47" t="str">
         <v>تم التحقق</v>
@@ -1929,7 +1929,7 @@
         <v>تحديد ما يحدث عند تعطل النظام أو إيقافه، بما في ذلك وجود بديل يدوي أو غير معتمد على الذكاء الاصطناعي، لضمان استمرار الخدمة بأمان.</v>
       </c>
       <c r="E48" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 8.2; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 2.1, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 8.2; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.4.2, 2.4.3; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 2.1, MEASURE 2.6; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15</v>
       </c>
       <c r="F48" t="str">
         <v>تم التحقق</v>
@@ -2025,7 +2025,7 @@
         <v>قبل الإطلاق وبعد كل تغيير جوهري، يُكلَّف أشخاص لم يشاركوا في بناء النظام بمحاولة دفعه إلى سلوك غير مقصود: محاولات كسر القيود، وحقن الأوامر المباشر وغير المباشر (بما في ذلك عبر المستندات أو الرسائل أو صفحات الويب التي يقرؤها)، واستخراج البيانات السرية، وإساءة استخدام أدواته. وتُوثَّق النتائج وتُعالَج ثم يُعاد الاختبار.</v>
       </c>
       <c r="E51" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 1.3, MEASURE 2.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 55</v>
+        <v>السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.5.2; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.6.2.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 1.3, MEASURE 2.6, MEASURE 2.7; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 55</v>
       </c>
       <c r="F51" t="str">
         <v>تم التحقق</v>
@@ -2057,7 +2057,7 @@
         <v>الاحتفاظ بقائمة بالنماذج ومجموعات البيانات ومكتبات الذكاء الاصطناعي التي يعتمد عليها النظام، مع مصدر كل منها وإصداره وترخيصه. وعدم الحصول عليها إلا من مصادر موثوقة، والتحقق من سلامتها قبل الاستخدام، وتثبيت إصداراتها، ومتابعة ثغراتها وتحديثاتها من المصدر، حتى لا يصل إلى بيئة التشغيل مكوّن جرى العبث به أو تحديثه دون علم.</v>
       </c>
       <c r="E52" t="str">
-        <v>أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.10.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MAP 4.1, MANAGE 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 25</v>
+        <v>السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.1.3; أخلاقيات الذكاء الاصطناعي في دبي: Security; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Privacy &amp; Security; آيزو/آي إي سي 42001: A.4.4, A.10.3; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: GOVERN 6.1, MAP 4.1, MANAGE 3.2; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 15, Art. 25</v>
       </c>
       <c r="F52" t="str">
         <v>تم التحقق</v>
@@ -2089,7 +2089,7 @@
         <v>مراقبة أداء النظام أثناء التشغيل وفق مؤشرات متفق عليها، وتحديد حدود التنبيه مسبقًا، وإسناد كل تنبيه إلى شخص مسؤول عن الاستجابة له.</v>
       </c>
       <c r="E53" t="str">
-        <v>كود الإمارات للخدمات الحكومية: Code 2.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 4.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26, Art. 72</v>
+        <v>كود الإمارات للخدمات الحكومية: Code 2.1; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.6.1; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Accountability &amp; Responsibility, Reliability &amp; Safety; آيزو/آي إي سي 42001: A.6.2.6; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MEASURE 2.4, MANAGE 4.1; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 26, Art. 72</v>
       </c>
       <c r="F53" t="str">
         <v>تم التحقق</v>
@@ -2185,7 +2185,7 @@
         <v>تحديد آلية الإبلاغ عن حوادث الذكاء الاصطناعي والأخطاء الجسيمة والتحقيق فيها ومعالجتها وإبلاغ المتأثرين بها، والجهات التنظيمية عند الاقتضاء.</v>
       </c>
       <c r="E56" t="str">
-        <v>مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 4.3, MANAGE 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 73</v>
+        <v>قانون حماية البيانات الشخصية: Art. 9; السياسة الوطنية للأمن السيبراني للذكاء الاصطناعي: 2.6.2, 2.6.3; مبادئ أخلاقيات الذكاء الاصطناعي (سدايا): Transparency &amp; Explainability; آيزو/آي إي سي 42001: A.8.4; إطار NIST لإدارة مخاطر الذكاء الاصطناعي: MANAGE 4.3, MANAGE 2.3; قانون الاتحاد الأوروبي للذكاء الاصطناعي: Art. 73</v>
       </c>
       <c r="F56" t="str">
         <v>تم التحقق</v>

</xml_diff>